<commit_message>
Update benchmark workbook compatibility
</commit_message>
<xml_diff>
--- a/benchmarks/negative_reconstruction/ground_truth.xlsx
+++ b/benchmarks/negative_reconstruction/ground_truth.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="ground_truth" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ground_truth'!$A$1:$J$483</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -642,7 +640,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -2252,7 +2250,7 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -2350,7 +2348,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -2886,7 +2884,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -2939,7 +2937,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -2992,7 +2990,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -3541,7 +3539,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -3590,7 +3588,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -3630,7 +3628,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -3738,7 +3736,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -3886,7 +3884,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -4663,7 +4661,7 @@
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
@@ -4718,7 +4716,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -4807,7 +4805,7 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
@@ -5352,7 +5350,7 @@
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
@@ -5541,7 +5539,7 @@
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G104" s="3" t="inlineStr">
@@ -6039,7 +6037,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -6488,7 +6486,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -7222,7 +7220,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -7980,7 +7978,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -8031,7 +8029,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -8082,7 +8080,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -8133,7 +8131,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -8282,7 +8280,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -8333,7 +8331,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -8384,7 +8382,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -9234,7 +9232,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -10789,7 +10787,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -10836,7 +10834,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -10883,7 +10881,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -11168,7 +11166,7 @@
       </c>
       <c r="F219" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G219" s="3" t="inlineStr">
@@ -12391,7 +12389,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -12436,7 +12434,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -12801,7 +12799,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -12851,7 +12849,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -12901,7 +12899,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -12951,7 +12949,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -13001,7 +12999,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -13051,7 +13049,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -13101,7 +13099,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -13151,7 +13149,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -13201,7 +13199,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -13251,7 +13249,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -13302,7 +13300,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -13353,7 +13351,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -13404,7 +13402,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -13455,7 +13453,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -13506,7 +13504,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -13557,7 +13555,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -13608,7 +13606,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">
@@ -13659,7 +13657,7 @@
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G270" s="2" t="inlineStr">
@@ -13710,7 +13708,7 @@
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G271" s="2" t="inlineStr">
@@ -13761,7 +13759,7 @@
       </c>
       <c r="F272" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G272" s="2" t="inlineStr">
@@ -13813,7 +13811,7 @@
       </c>
       <c r="F273" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G273" s="2" t="inlineStr">
@@ -13865,7 +13863,7 @@
       </c>
       <c r="F274" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G274" s="2" t="inlineStr">
@@ -13917,7 +13915,7 @@
       </c>
       <c r="F275" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G275" s="2" t="inlineStr">
@@ -13969,7 +13967,7 @@
       </c>
       <c r="F276" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G276" s="2" t="inlineStr">
@@ -14021,7 +14019,7 @@
       </c>
       <c r="F277" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G277" s="2" t="inlineStr">
@@ -14074,7 +14072,7 @@
       </c>
       <c r="F278" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G278" s="2" t="inlineStr">
@@ -14456,7 +14454,7 @@
       </c>
       <c r="F285" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G285" s="2" t="inlineStr">
@@ -14512,7 +14510,7 @@
       </c>
       <c r="F286" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G286" s="2" t="inlineStr">
@@ -14568,7 +14566,7 @@
       </c>
       <c r="F287" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G287" s="2" t="inlineStr">
@@ -14622,7 +14620,7 @@
       </c>
       <c r="F288" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G288" s="2" t="inlineStr">
@@ -14676,7 +14674,7 @@
       </c>
       <c r="F289" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G289" s="2" t="inlineStr">
@@ -14730,7 +14728,7 @@
       </c>
       <c r="F290" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G290" s="2" t="inlineStr">
@@ -14784,7 +14782,7 @@
       </c>
       <c r="F291" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G291" s="2" t="inlineStr">
@@ -14838,7 +14836,7 @@
       </c>
       <c r="F292" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G292" s="2" t="inlineStr">
@@ -15115,7 +15113,7 @@
       </c>
       <c r="F297" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G297" s="2" t="inlineStr">
@@ -15171,7 +15169,7 @@
       </c>
       <c r="F298" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G298" s="2" t="inlineStr">
@@ -15227,7 +15225,7 @@
       </c>
       <c r="F299" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G299" s="2" t="inlineStr">
@@ -15282,7 +15280,7 @@
       </c>
       <c r="F300" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G300" s="2" t="inlineStr">
@@ -15629,7 +15627,7 @@
       </c>
       <c r="F307" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G307" s="2" t="inlineStr">
@@ -15684,7 +15682,7 @@
       </c>
       <c r="F308" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G308" s="2" t="inlineStr">
@@ -15739,7 +15737,7 @@
       </c>
       <c r="F309" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G309" s="2" t="inlineStr">
@@ -15788,7 +15786,7 @@
       </c>
       <c r="F310" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G310" s="2" t="inlineStr">
@@ -15837,7 +15835,7 @@
       </c>
       <c r="F311" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G311" s="2" t="inlineStr">
@@ -15892,7 +15890,7 @@
       </c>
       <c r="F312" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G312" s="2" t="inlineStr">
@@ -15947,7 +15945,7 @@
       </c>
       <c r="F313" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G313" s="2" t="inlineStr">
@@ -15996,7 +15994,7 @@
       </c>
       <c r="F314" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G314" s="2" t="inlineStr">
@@ -16036,7 +16034,7 @@
       </c>
       <c r="F315" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G315" s="3" t="inlineStr">
@@ -16076,7 +16074,7 @@
       </c>
       <c r="F316" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G316" s="3" t="inlineStr">
@@ -16323,7 +16321,7 @@
       </c>
       <c r="F321" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G321" s="2" t="inlineStr">
@@ -16934,7 +16932,7 @@
       </c>
       <c r="F333" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G333" s="2" t="inlineStr">
@@ -17096,7 +17094,7 @@
       </c>
       <c r="F336" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G336" s="2" t="inlineStr">
@@ -18319,7 +18317,7 @@
       </c>
       <c r="F362" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G362" s="2" t="inlineStr">
@@ -18369,7 +18367,7 @@
       </c>
       <c r="F363" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G363" s="2" t="inlineStr">
@@ -18419,7 +18417,7 @@
       </c>
       <c r="F364" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G364" s="2" t="inlineStr">
@@ -18459,7 +18457,7 @@
       </c>
       <c r="F365" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G365" s="3" t="inlineStr">
@@ -18799,7 +18797,7 @@
       </c>
       <c r="F372" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G372" s="3" t="inlineStr">
@@ -18839,7 +18837,7 @@
       </c>
       <c r="F373" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G373" s="3" t="inlineStr">
@@ -19454,7 +19452,7 @@
       </c>
       <c r="F386" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G386" s="3" t="inlineStr">
@@ -19504,7 +19502,7 @@
       </c>
       <c r="F387" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G387" s="2" t="inlineStr">
@@ -20177,7 +20175,7 @@
       </c>
       <c r="F401" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G401" s="2" t="inlineStr">
@@ -20276,7 +20274,7 @@
       </c>
       <c r="F403" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G403" s="2" t="inlineStr">
@@ -20326,7 +20324,7 @@
       </c>
       <c r="F404" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G404" s="2" t="inlineStr">
@@ -20474,7 +20472,7 @@
       </c>
       <c r="F407" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G407" s="2" t="inlineStr">
@@ -20885,7 +20883,7 @@
       </c>
       <c r="F416" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G416" s="2" t="inlineStr">
@@ -21132,7 +21130,7 @@
       </c>
       <c r="F421" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G421" s="2" t="inlineStr">
@@ -24152,7 +24150,7 @@
       </c>
       <c r="F483" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G483" s="3" t="inlineStr">
@@ -24173,7 +24171,6 @@
       <c r="J483" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J483"/>
   <dataValidations count="1">
     <dataValidation sqref="F2:I483" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Choose Yes or No" error="Select Yes or No for annotator contribution." type="list">
       <formula1>"Yes,No"</formula1>

</xml_diff>

<commit_message>
Add annotator comments to negative reference
Fill "Optional: comment by contributing annotator" for 100 rows
(58 evidence passages, papers N001-N032) with A1's evidence notes.
No other cells, the embedded matching data, or scores change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmarks/negative_reconstruction/ground_truth.xlsx
+++ b/benchmarks/negative_reconstruction/ground_truth.xlsx
@@ -569,7 +569,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>described mixture without FA yielding unidentified phase</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -618,7 +622,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>described mixture without FA yielding unidentified phase</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="38" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -707,7 +715,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>stated addition of na2wo4 is essential, crysatline pyproducts without it</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -757,7 +769,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>ph below listed gives clear solution ph above give amorphous solid</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -807,7 +823,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>ph below listed gives clear solution ph above give amorphous solid</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -856,7 +876,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>stated addition of na2wo4 is essential, crysatline pyproducts without it</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -906,7 +930,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>ph below listed gives clear solution ph above give amorphous solid</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -956,7 +984,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>ph below listed gives clear solution ph above give amorphous solid</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1006,7 +1038,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>many attemps with replacements for CuI and Et4NI did not afford the desired compount 2</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1056,7 +1092,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>many attemps with replacements for CuI and Et4NI did not afford the desired compount 2</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -1105,7 +1145,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>many attemps with replacements for CuI and Et4NI did not afford the desired compount 2</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1154,7 +1198,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -1203,7 +1251,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1252,7 +1304,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J16" s="2" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -1301,7 +1357,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J17" s="2" t="n"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1350,7 +1410,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J18" s="2" t="n"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -1399,7 +1463,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J19" s="2" t="n"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -1448,7 +1516,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J20" s="2" t="n"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -1497,7 +1569,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J21" s="2" t="n"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -1546,7 +1622,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J22" s="2" t="n"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -1595,7 +1675,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J23" s="2" t="n"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="45" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -1644,7 +1728,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J24" s="2" t="n"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="45" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -1693,7 +1781,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J25" s="2" t="n"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="45" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -1742,7 +1834,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J26" s="2" t="n"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="45" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -1791,7 +1887,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J27" s="2" t="n"/>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -1840,7 +1940,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J28" s="2" t="n"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="45" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
@@ -1889,7 +1993,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J29" s="2" t="n"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -1938,7 +2046,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J30" s="2" t="n"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
@@ -1987,7 +2099,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J31" s="2" t="n"/>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>when the desired temp is changed by more than 15 C the desired compounds cannot be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="45" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -2036,7 +2152,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J32" s="2" t="n"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>said cannot obtain target compounds without hcooh</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
@@ -2085,7 +2205,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J33" s="2" t="n"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>said cannot obtain target compounds without hcooh</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="45" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -2134,7 +2258,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J34" s="2" t="n"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>when changing agch3coo to agno3 no crystals were obtained</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="45" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
@@ -2179,7 +2307,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J35" s="2" t="n"/>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>paper says none of the cuII mofs are acceibly through traditional one pot synthesis</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="45" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -2228,7 +2360,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J36" s="2" t="n"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>paper says none of the cuII mofs are acceibly through traditional one pot synthesis</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="38" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
@@ -2317,7 +2453,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J38" s="2" t="n"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>paper says without modulating agent get broad pxrd reflections, low crysatlinity</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="45" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
@@ -2366,7 +2506,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J39" s="2" t="n"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>tabl one has large screening data shwoing failed attempts</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="135" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
@@ -2421,7 +2565,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J40" s="2" t="n"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>tabl one has large screening data shwoing failed attempts</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="135" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
@@ -2476,7 +2624,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J41" s="2" t="n"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>tabl one has large screening data shwoing failed attempts</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="135" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -2531,7 +2683,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J42" s="2" t="n"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>tabl one has large screening data shwoing failed attempts</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="105" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
@@ -2584,7 +2740,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J43" s="2" t="n"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>tabl one has large screening data shwoing failed attempts</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="105" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -2637,7 +2797,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J44" s="2" t="n"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>tabl one has large screening data shwoing failed attempts</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="105" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
@@ -2690,7 +2854,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J45" s="2" t="n"/>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>tabl one has large screening data shwoing failed attempts</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="105" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
@@ -2743,7 +2911,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J46" s="2" t="n"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>tabl one has large screening data shwoing failed attempts</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="105" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
@@ -2796,7 +2968,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J47" s="2" t="n"/>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>tabl one has large screening data shwoing failed attempts</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="105" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
@@ -2849,7 +3025,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J48" s="2" t="n"/>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>tabl one has large screening data shwoing failed attempts</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="105" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
@@ -2902,7 +3082,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J49" s="2" t="n"/>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>large screening table with negatives as table 1</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="105" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
@@ -2955,7 +3139,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J50" s="2" t="n"/>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>large screening table with negatives as table 1</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="105" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
@@ -3008,7 +3196,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J51" s="2" t="n"/>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>large screening table with negatives as table 1</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="45" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
@@ -3057,7 +3249,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J52" s="2" t="n"/>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>paper says synthesis fails wuthout metal ions or with sodium salts isntead of iron</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="45" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
@@ -3106,7 +3302,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J53" s="2" t="n"/>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>paper says synthesis fails wuthout metal ions or with sodium salts isntead of iron</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="75" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
@@ -3157,7 +3357,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J54" s="2" t="n"/>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>paper says ordered structure would be destroyed by excessive dilution of mof precursor</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="45" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
@@ -3206,7 +3410,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J55" s="2" t="n"/>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>papers says if non optiomal conditions are observed, xray amorphous solids form</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="45" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
@@ -3255,7 +3463,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J56" s="2" t="n"/>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>papers says if non optiomal conditions are observed, xray amorphous solids form</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="45" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
@@ -3304,7 +3516,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J57" s="2" t="n"/>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>papers says if non optiomal conditions are observed, xray amorphous solids form</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="60" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
@@ -3354,7 +3570,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J58" s="2" t="n"/>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>papers says if non optiomal conditions are observed, xray amorphous solids form</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="60" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
@@ -3404,7 +3624,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J59" s="2" t="n"/>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>papers says if non optiomal conditions are observed, xray amorphous solids form</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="60" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
@@ -3454,7 +3678,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J60" s="2" t="n"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>papers says if non optiomal conditions are observed, xray amorphous solids form</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="90" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
@@ -3506,7 +3734,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J61" s="2" t="n"/>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>papers says if non optiomal conditions are observed, xray amorphous solids form</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="75" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
@@ -3557,7 +3789,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J62" s="2" t="n"/>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>papers says if non optiomal conditions are observed, xray amorphous solids form</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="45" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
@@ -3606,7 +3842,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J63" s="2" t="n"/>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>papers says if non optiomal conditions are observed, xray amorphous solids form</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="38" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
@@ -3704,7 +3944,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J65" s="2" t="n"/>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>paper says cuI reaction with l2 gives no product</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="60" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
@@ -3754,7 +3998,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J66" s="2" t="n"/>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>paper says cuI reaction with l2 gives no product</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="45" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
@@ -3803,7 +4051,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J67" s="2" t="n"/>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>fig captions say that znso47h20 gives unknown and no product is made with zlcl2</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="45" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
@@ -3852,7 +4104,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J68" s="2" t="n"/>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>fig captions say that znso47h20 gives unknown and no product is made with zlcl2</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="60" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
@@ -3902,7 +4158,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J69" s="2" t="n"/>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>paper says wthat with added water the mof-5 doesn’t form</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="45" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
@@ -3951,7 +4211,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J70" s="2" t="n"/>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>papers describeds lot of solvents as giving unknown phases</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="45" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
@@ -4000,7 +4264,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J71" s="2" t="n"/>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>papers describeds lot of solvents as giving unknown phases</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="45" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
@@ -4049,7 +4317,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J72" s="2" t="n"/>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>gives conditions and says no solid product detected</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="45" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
@@ -4098,7 +4370,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J73" s="2" t="n"/>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>gives conditions and says no solid product detected</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="45" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
@@ -4147,7 +4423,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J74" s="2" t="n"/>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>describes conditions and says gave xray amorphous solids</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="45" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
@@ -4196,7 +4476,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J75" s="2" t="n"/>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>says at higher concentrations mof and crystaline byproduct are formed</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="45" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
@@ -4245,7 +4529,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J76" s="2" t="n"/>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>says higher temps result in more crystaline products</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="45" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
@@ -4294,7 +4582,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J77" s="2" t="n"/>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>says without addition of modulator amorphous phase obtained</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="45" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
@@ -4343,7 +4635,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J78" s="2" t="n"/>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>control experiments ran without bipyridine ligands and failed to obtain</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="60" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
@@ -4393,7 +4689,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J79" s="2" t="n"/>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>lists specific pHs and says were unable to obtain satisfactor products</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="60" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
@@ -4443,7 +4743,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J80" s="2" t="n"/>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>lists specific pHs and says attempts to synthesize mof also failed</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="45" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
@@ -4492,7 +4796,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J81" s="2" t="n"/>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>lists lots of linkers then says only 1 worked</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="45" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
@@ -4541,7 +4849,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J82" s="2" t="n"/>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>lists lots of linkers then says only 1 worked</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="45" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
@@ -4590,7 +4902,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J83" s="2" t="n"/>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>lists lots of linkers then says only 1 worked</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="45" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
@@ -4639,7 +4955,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J84" s="2" t="n"/>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>conventional synthesis of two reagents in water at room temp led to an amorphous phase</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="38" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
@@ -4734,7 +5054,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J86" s="2" t="n"/>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>acetic acid amount screenings figure</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="45" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
@@ -4783,7 +5107,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J87" s="2" t="n"/>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>says control experiments carried out w/ no water or in water/dmf did not afford crystaline materials</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="38" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
@@ -4868,7 +5196,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J89" s="2" t="n"/>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>said that aniline and imidazole worked after"several trails using other N containing ligands</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="45" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
@@ -4913,7 +5245,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J90" s="2" t="n"/>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>said that aniline and imidazole worked after"several trails using other N containing ligands</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="45" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
@@ -4958,7 +5294,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J91" s="2" t="n"/>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>said that aniline and imidazole worked after"several trails using other N containing ligands</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="75" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
@@ -5144,7 +5484,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J95" s="2" t="n"/>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>said that aniline and imidazole worked after"several trails using other N containing ligands</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="45" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
@@ -5189,7 +5533,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J96" s="2" t="n"/>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>said that aniline and imidazole worked after"several trails using other N containing ligands</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="45" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
@@ -5234,7 +5582,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J97" s="2" t="n"/>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>said that aniline and imidazole worked after"several trails using other N containing ligands</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="45" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
@@ -5279,7 +5631,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J98" s="2" t="n"/>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>lists molar ratio and solvent changes as attepted previous conditions</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="45" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
@@ -5328,7 +5684,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J99" s="2" t="n"/>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>says that attempts to synthesis mof with same conditions but no pyrazole failed</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="38" customHeight="1">
       <c r="A100" s="3" t="inlineStr">
@@ -5417,7 +5777,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J101" s="2" t="n"/>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>says other amorphous unidentified crysatline phases were obtained for Er, Yb and Ce</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="60" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
@@ -5467,7 +5831,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J102" s="2" t="n"/>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>says other amorphous unidentified crysatline phases were obtained for Er, Yb and Ce</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="60" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
@@ -5517,7 +5885,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J103" s="2" t="n"/>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>says other amorphous unidentified crysatline phases were obtained for Er, Yb and Ce</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="38" customHeight="1">
       <c r="A104" s="3" t="inlineStr">
@@ -5606,7 +5978,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J105" s="2" t="n"/>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>screening table s3 shows amorphous without modulator</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="45" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
@@ -5655,7 +6031,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J106" s="2" t="n"/>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>says with no additive or with hcl gets prooly crystaline phase</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="45" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
@@ -5704,7 +6084,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J107" s="2" t="n"/>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>says with no additive or with hcl gets prooly crystaline phase</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="60" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
@@ -5804,7 +6188,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J109" s="2" t="n"/>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>described dramatically lower yield using nitrate salts instead of acetate salts</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="60" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
@@ -5854,7 +6242,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J110" s="2" t="n"/>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>says nitrate salts yiled low porosity and low yield</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="45" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
@@ -5903,7 +6295,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J111" s="2" t="n"/>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>says nitrate salts yiled low porosity and low yield</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="60" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
@@ -6004,7 +6400,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J113" s="2" t="n"/>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>says nitrate salts yiled low porosity and low yield</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="75" customHeight="1">
       <c r="A114" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Fill annotator comments for all negative reference rows
Fill "Optional: comment by contributing annotator" for the remaining
367 rows (all 100 papers now have A1's evidence notes on every scored
and optional row) and update 3 earlier comments that A1 revised.
No other cells, the embedded matching data, or scores change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmarks/negative_reconstruction/ground_truth.xlsx
+++ b/benchmarks/negative_reconstruction/ground_truth.xlsx
@@ -1147,7 +1147,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>many attemps with replacements for CuI and Et4NI did not afford the desired compount 2</t>
+          <t>many attemps without et4ni fialed to give compount 2</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4160,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>paper says wthat with added water the mof-5 doesn’t form</t>
+          <t>mixtures with high conent of mesitylene do not lead to the formation of mof-5</t>
         </is>
       </c>
     </row>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>says higher temps result in more crystaline products</t>
+          <t>says higher temps result in less crystaline products</t>
         </is>
       </c>
     </row>
@@ -5345,7 +5345,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J92" s="2" t="n"/>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>different molar ratios and solvents were tried before adding aniline</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="75" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
@@ -5392,7 +5396,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J93" s="2" t="n"/>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>different molar ratios and solvents were tried before adding aniline</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="75" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
@@ -5439,7 +5447,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J94" s="2" t="n"/>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>different molar ratios and solvents were tried before adding aniline</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="45" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
@@ -6138,7 +6150,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J108" s="2" t="n"/>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>bpdc version has broad brdpeaks and low Bet</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="60" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
@@ -6349,7 +6365,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J112" s="2" t="n"/>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>bpdc version has broad brdpeaks and low Bet</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="75" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
@@ -6455,7 +6475,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J114" s="2" t="n"/>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>.5 h product had low porosity, irregular morphologie and low yield</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="60" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
@@ -6505,7 +6529,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J115" s="2" t="n"/>
+      <c r="J115" s="2" t="inlineStr">
+        <is>
+          <t>table S8 reports no products</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="60" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
@@ -6555,7 +6583,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J116" s="2" t="n"/>
+      <c r="J116" s="2" t="inlineStr">
+        <is>
+          <t>with low bdc concentration low yield and crystalinity</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="45" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
@@ -6604,7 +6636,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J117" s="2" t="n"/>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>.5 M Can was a liquid sate during the reaction time, and uio-66ce could not be obtained under a low concentration of can</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="45" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
@@ -6653,7 +6689,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J118" s="2" t="n"/>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>.5 M Can was a liquid sate during the reaction time, and uio-66ce could not be obtained under a low concentration of can</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="60" customHeight="1">
       <c r="A119" s="2" t="inlineStr">
@@ -6703,7 +6743,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J119" s="2" t="n"/>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
+          <t>paper says it was clear uio-66 could hardly be produced in DMF</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="75" customHeight="1">
       <c r="A120" s="2" t="inlineStr">
@@ -6754,7 +6798,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J120" s="2" t="n"/>
+      <c r="J120" s="2" t="inlineStr">
+        <is>
+          <t>bad ramman peaks when using aqueous solution</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="45" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
@@ -6803,7 +6851,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J121" s="2" t="n"/>
+      <c r="J121" s="2" t="inlineStr">
+        <is>
+          <t>at 1.0M naoh of hcl no product obtained</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="45" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
@@ -6852,7 +6904,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J122" s="2" t="n"/>
+      <c r="J122" s="2" t="inlineStr">
+        <is>
+          <t>at 1.0M naoh of hcl no product obtained</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="90" customHeight="1">
       <c r="A123" s="2" t="inlineStr">
@@ -6904,7 +6960,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J123" s="2" t="n"/>
+      <c r="J123" s="2" t="inlineStr">
+        <is>
+          <t>BHC only gave clear solutions under solvothermal conditions</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="90" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
@@ -6956,7 +7016,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J124" s="2" t="n"/>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>could not be synthesies via tradiotnal solvothermal approach</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="90" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
@@ -7008,7 +7072,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J125" s="2" t="n"/>
+      <c r="J125" s="2" t="inlineStr">
+        <is>
+          <t>could not be synthesies via tradiotnal solvothermal approach</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="45" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
@@ -7057,7 +7125,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J126" s="2" t="n"/>
+      <c r="J126" s="2" t="inlineStr">
+        <is>
+          <t>table 1 reports no rystals</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="60" customHeight="1">
       <c r="A127" s="2" t="inlineStr">
@@ -7107,7 +7179,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J127" s="2" t="n"/>
+      <c r="J127" s="2" t="inlineStr">
+        <is>
+          <t>formed but with greatly reduced yield</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="45" customHeight="1">
       <c r="A128" s="2" t="inlineStr">
@@ -7156,7 +7232,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J128" s="2" t="n"/>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
+          <t>MAF forms with low crystalinity ( no template)</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="45" customHeight="1">
       <c r="A129" s="2" t="inlineStr">
@@ -7201,7 +7281,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J129" s="2" t="n"/>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
+          <t>apparent at 10 equiv of naoh inorganic products are more common</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="45" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
@@ -7246,7 +7330,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J130" s="2" t="n"/>
+      <c r="J130" s="2" t="inlineStr">
+        <is>
+          <t>apparent at 10 equiv of naoh inorganic products are more common</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="45" customHeight="1">
       <c r="A131" s="2" t="inlineStr">
@@ -7295,7 +7383,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J131" s="2" t="n"/>
+      <c r="J131" s="2" t="inlineStr">
+        <is>
+          <t>says the use of 5 membered rings as guests wwre unseccessful and no product was formed</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="45" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
@@ -7344,7 +7436,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J132" s="2" t="n"/>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>says the use of 5 membered rings as guests wwre unseccessful and no product was formed</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="45" customHeight="1">
       <c r="A133" s="2" t="inlineStr">
@@ -7393,7 +7489,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J133" s="2" t="n"/>
+      <c r="J133" s="2" t="inlineStr">
+        <is>
+          <t>says the use of 5 membered rings as guests wwre unseccessful and no product was formed</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="45" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
@@ -7442,7 +7542,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J134" s="2" t="n"/>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
+          <t>presence of guest molecules(modulators)  was a key condition for synthesis with LN3</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="45" customHeight="1">
       <c r="A135" s="2" t="inlineStr">
@@ -7491,7 +7595,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J135" s="2" t="n"/>
+      <c r="J135" s="2" t="inlineStr">
+        <is>
+          <t>says the use of 5 membered rings as guests wwre unseccessful and no product was formed</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="45" customHeight="1">
       <c r="A136" s="2" t="inlineStr">
@@ -7540,7 +7648,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J136" s="2" t="n"/>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>says the use of 5 membered rings as guests wwre unseccessful and no product was formed</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="45" customHeight="1">
       <c r="A137" s="2" t="inlineStr">
@@ -7589,7 +7701,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J137" s="2" t="n"/>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>says the use of 5 membered rings as guests wwre unseccessful and no product was formed</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="45" customHeight="1">
       <c r="A138" s="2" t="inlineStr">
@@ -7638,7 +7754,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J138" s="2" t="n"/>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
+          <t>presence of guest molecules(modulators)  was a key condition for synthesis with LN3</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="45" customHeight="1">
       <c r="A139" s="2" t="inlineStr">
@@ -7687,7 +7807,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J139" s="2" t="n"/>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>the homologous gold compound of 3.h2o cannot form, no gold version</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="75" customHeight="1">
       <c r="A140" s="2" t="inlineStr">
@@ -7738,7 +7862,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J140" s="2" t="n"/>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>a list of mods temps and times are given and only a specific few are said to work</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="75" customHeight="1">
       <c r="A141" s="2" t="inlineStr">
@@ -7789,7 +7917,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J141" s="2" t="n"/>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>a list of mods temps and times are given and only a specific few are said to work</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="75" customHeight="1">
       <c r="A142" s="2" t="inlineStr">
@@ -7840,7 +7972,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J142" s="2" t="n"/>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>a list of mods temps and times are given and only a specific few are said to work</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="75" customHeight="1">
       <c r="A143" s="2" t="inlineStr">
@@ -7891,7 +8027,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J143" s="2" t="n"/>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>a list of mods temps and times are given and only a specific few are said to work</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="75" customHeight="1">
       <c r="A144" s="2" t="inlineStr">
@@ -7942,7 +8082,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J144" s="2" t="n"/>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>a list of mods temps and times are given and only a specific few are said to work</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="75" customHeight="1">
       <c r="A145" s="2" t="inlineStr">
@@ -7993,7 +8137,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J145" s="2" t="n"/>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>a list of mods temps and times are given and only a specific few are said to work</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="75" customHeight="1">
       <c r="A146" s="2" t="inlineStr">
@@ -8044,7 +8192,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J146" s="2" t="n"/>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
+          <t>a list of mods temps and times are given and only a specific few are said to work</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="75" customHeight="1">
       <c r="A147" s="2" t="inlineStr">
@@ -8095,7 +8247,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J147" s="2" t="n"/>
+      <c r="J147" s="2" t="inlineStr">
+        <is>
+          <t>a list of mods temps and times are given and only a specific few are said to work</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="75" customHeight="1">
       <c r="A148" s="2" t="inlineStr">
@@ -8146,7 +8302,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J148" s="2" t="n"/>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>a list of mods temps and times are given and only a specific few are said to work</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="60" customHeight="1">
       <c r="A149" s="2" t="inlineStr">
@@ -8196,7 +8356,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J149" s="2" t="n"/>
+      <c r="J149" s="2" t="inlineStr">
+        <is>
+          <t>a list of mods temps and times are given and only a specific few are said to work</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="60" customHeight="1">
       <c r="A150" s="2" t="inlineStr">
@@ -8246,7 +8410,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J150" s="2" t="n"/>
+      <c r="J150" s="2" t="inlineStr">
+        <is>
+          <t>a list of mods temps and times are given and only a specific few are said to work</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="60" customHeight="1">
       <c r="A151" s="2" t="inlineStr">
@@ -8296,7 +8464,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J151" s="2" t="n"/>
+      <c r="J151" s="2" t="inlineStr">
+        <is>
+          <t>prolonged experiments with 120 equiv for 10 days yieldied clear solution</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="45" customHeight="1">
       <c r="A152" s="2" t="inlineStr">
@@ -8345,7 +8517,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J152" s="2" t="n"/>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>was not able to isolate a crystline framework from the gel produced with these conditions</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="75" customHeight="1">
       <c r="A153" s="2" t="inlineStr">
@@ -8396,7 +8572,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J153" s="2" t="n"/>
+      <c r="J153" s="2" t="inlineStr">
+        <is>
+          <t>isolated product after 3 hours had amorphoues fe3o bpdc</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="75" customHeight="1">
       <c r="A154" s="2" t="inlineStr">
@@ -8447,7 +8627,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J154" s="2" t="n"/>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>isolated product after 3 hours had amorphoues fe2cro bpdc</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="75" customHeight="1">
       <c r="A155" s="2" t="inlineStr">
@@ -8498,7 +8682,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J155" s="2" t="n"/>
+      <c r="J155" s="2" t="inlineStr">
+        <is>
+          <t>si fig s32 shows mateirl ioalated after 3 h reactio not crystalized</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="75" customHeight="1">
       <c r="A156" s="2" t="inlineStr">
@@ -8549,7 +8737,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J156" s="2" t="n"/>
+      <c r="J156" s="2" t="inlineStr">
+        <is>
+          <t>si fig s30 shows mateirl ioalated after 3 h reactio not crystalized</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="45" customHeight="1">
       <c r="A157" s="2" t="inlineStr">
@@ -8598,7 +8790,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J157" s="2" t="n"/>
+      <c r="J157" s="2" t="inlineStr">
+        <is>
+          <t>pxrd for cr containing materials show gelation rather than crystalization</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="45" customHeight="1">
       <c r="A158" s="2" t="inlineStr">
@@ -8647,7 +8843,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J158" s="2" t="n"/>
+      <c r="J158" s="2" t="inlineStr">
+        <is>
+          <t>pxrd for cr containing materials show gelation rather than crystalization</t>
+        </is>
+      </c>
     </row>
     <row r="159" ht="75" customHeight="1">
       <c r="A159" s="2" t="inlineStr">
@@ -8698,7 +8898,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J159" s="2" t="n"/>
+      <c r="J159" s="2" t="inlineStr">
+        <is>
+          <t>3h isolated product still in gel phase pre crystal</t>
+        </is>
+      </c>
     </row>
     <row r="160" ht="75" customHeight="1">
       <c r="A160" s="2" t="inlineStr">
@@ -8749,7 +8953,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J160" s="2" t="n"/>
+      <c r="J160" s="2" t="inlineStr">
+        <is>
+          <t>3h isolated product still in gel phase pre crystal</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="75" customHeight="1">
       <c r="A161" s="2" t="inlineStr">
@@ -8800,7 +9008,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J161" s="2" t="n"/>
+      <c r="J161" s="2" t="inlineStr">
+        <is>
+          <t>3h isolated product still in gel phase pre crystal</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="45" customHeight="1">
       <c r="A162" s="2" t="inlineStr">
@@ -8849,7 +9061,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J162" s="2" t="n"/>
+      <c r="J162" s="2" t="inlineStr">
+        <is>
+          <t>pxrd for cr containing materials show gelation rather than crystalization</t>
+        </is>
+      </c>
     </row>
     <row r="163" ht="75" customHeight="1">
       <c r="A163" s="2" t="inlineStr">
@@ -8900,7 +9116,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J163" s="2" t="n"/>
+      <c r="J163" s="2" t="inlineStr">
+        <is>
+          <t>SI table show screening conditions with amrphpus or unknown products</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="75" customHeight="1">
       <c r="A164" s="2" t="inlineStr">
@@ -8951,7 +9171,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J164" s="2" t="n"/>
+      <c r="J164" s="2" t="inlineStr">
+        <is>
+          <t>SI table show screening conditions with amrphpus or unknown products</t>
+        </is>
+      </c>
     </row>
     <row r="165" ht="75" customHeight="1">
       <c r="A165" s="2" t="inlineStr">
@@ -9002,7 +9226,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J165" s="2" t="n"/>
+      <c r="J165" s="2" t="inlineStr">
+        <is>
+          <t>SI table show screening conditions with amrphpus or unknown products</t>
+        </is>
+      </c>
     </row>
     <row r="166" ht="75" customHeight="1">
       <c r="A166" s="2" t="inlineStr">
@@ -9053,7 +9281,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J166" s="2" t="n"/>
+      <c r="J166" s="2" t="inlineStr">
+        <is>
+          <t>SI table show screening conditions with amrphpus or unknown products</t>
+        </is>
+      </c>
     </row>
     <row r="167" ht="75" customHeight="1">
       <c r="A167" s="2" t="inlineStr">
@@ -9104,7 +9336,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J167" s="2" t="n"/>
+      <c r="J167" s="2" t="inlineStr">
+        <is>
+          <t>SI table show screening conditions with amrphpus or unknown products</t>
+        </is>
+      </c>
     </row>
     <row r="168" ht="75" customHeight="1">
       <c r="A168" s="2" t="inlineStr">
@@ -9155,7 +9391,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J168" s="2" t="n"/>
+      <c r="J168" s="2" t="inlineStr">
+        <is>
+          <t>3 specific conditions are named with bad oxrd peaks indicating "lack of crystalization"</t>
+        </is>
+      </c>
     </row>
     <row r="169" ht="75" customHeight="1">
       <c r="A169" s="2" t="inlineStr">
@@ -9206,7 +9446,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J169" s="2" t="n"/>
+      <c r="J169" s="2" t="inlineStr">
+        <is>
+          <t>3 specific conditions are named with bad oxrd peaks indicating "lack of crystalization"</t>
+        </is>
+      </c>
     </row>
     <row r="170" ht="90" customHeight="1">
       <c r="A170" s="2" t="inlineStr">
@@ -9258,7 +9502,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J170" s="2" t="n"/>
+      <c r="J170" s="2" t="inlineStr">
+        <is>
+          <t>3 specific conditions are named with bad oxrd peaks indicating "lack of crystalization"</t>
+        </is>
+      </c>
     </row>
     <row r="171" ht="45" customHeight="1">
       <c r="A171" s="2" t="inlineStr">
@@ -9303,7 +9551,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J171" s="2" t="n"/>
+      <c r="J171" s="2" t="inlineStr">
+        <is>
+          <t>says cd/cpds complex is not succecedd or not suitible for single crssyal xrd</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="45" customHeight="1">
       <c r="A172" s="2" t="inlineStr">
@@ -9352,7 +9604,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J172" s="2" t="n"/>
+      <c r="J172" s="2" t="inlineStr">
+        <is>
+          <t>carrying out this reaction in methanol results in clkear solution</t>
+        </is>
+      </c>
     </row>
     <row r="173" ht="45" customHeight="1">
       <c r="A173" s="2" t="inlineStr">
@@ -9401,7 +9657,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J173" s="2" t="n"/>
+      <c r="J173" s="2" t="inlineStr">
+        <is>
+          <t>says NICS-4 did not form at longer crysalzation times, evenn at lower temp</t>
+        </is>
+      </c>
     </row>
     <row r="174" ht="45" customHeight="1">
       <c r="A174" s="2" t="inlineStr">
@@ -9450,7 +9710,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J174" s="2" t="n"/>
+      <c r="J174" s="2" t="inlineStr">
+        <is>
+          <t>says it only crysatlizeds in pure ethanol, and more options are shown in fig 11</t>
+        </is>
+      </c>
     </row>
     <row r="175" ht="60" customHeight="1">
       <c r="A175" s="2" t="inlineStr">
@@ -9500,7 +9764,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J175" s="2" t="n"/>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>says below a 1.33 ML ratio product was a solid phase rather than MOF</t>
+        </is>
+      </c>
     </row>
     <row r="176" ht="60" customHeight="1">
       <c r="A176" s="2" t="inlineStr">
@@ -9550,7 +9818,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J176" s="2" t="n"/>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>says at 120 C and below intermedaite phases persisted with an absensee of MOF-5</t>
+        </is>
+      </c>
     </row>
     <row r="177" ht="60" customHeight="1">
       <c r="A177" s="2" t="inlineStr">
@@ -9600,7 +9872,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J177" s="2" t="n"/>
+      <c r="J177" s="2" t="inlineStr">
+        <is>
+          <t>says at all temps no solid material is producted in the first 30 mins of heating</t>
+        </is>
+      </c>
     </row>
     <row r="178" ht="60" customHeight="1">
       <c r="A178" s="2" t="inlineStr">
@@ -9650,7 +9926,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J178" s="2" t="n"/>
+      <c r="J178" s="2" t="inlineStr">
+        <is>
+          <t>says at all temps no solid material is producted in the first 30 mins of heating</t>
+        </is>
+      </c>
     </row>
     <row r="179" ht="60" customHeight="1">
       <c r="A179" s="2" t="inlineStr">
@@ -9700,7 +9980,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J179" s="2" t="n"/>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>lists lots of attempted % solids then lists 20% and 30% as not working</t>
+        </is>
+      </c>
     </row>
     <row r="180" ht="60" customHeight="1">
       <c r="A180" s="2" t="inlineStr">
@@ -9750,7 +10034,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J180" s="2" t="n"/>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>lists lots of attempted % solids then lists 20% and 30% as not working</t>
+        </is>
+      </c>
     </row>
     <row r="181" ht="45" customHeight="1">
       <c r="A181" s="2" t="inlineStr">
@@ -9799,7 +10087,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J181" s="2" t="n"/>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>no solid materail produced in the first 30 mins of heating</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="75" customHeight="1">
       <c r="A182" s="2" t="inlineStr">
@@ -9850,7 +10142,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J182" s="2" t="n"/>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>listed many screening conditions attempted to find optimal conditons and solvent system was one of them</t>
+        </is>
+      </c>
     </row>
     <row r="183" ht="75" customHeight="1">
       <c r="A183" s="2" t="inlineStr">
@@ -9901,7 +10197,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J183" s="2" t="n"/>
+      <c r="J183" s="2" t="inlineStr">
+        <is>
+          <t>listed many screening conditions attempted to find optimal conditons and solvent system was one of them</t>
+        </is>
+      </c>
     </row>
     <row r="184" ht="75" customHeight="1">
       <c r="A184" s="2" t="inlineStr">
@@ -9952,7 +10252,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J184" s="2" t="n"/>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>listed many screening conditions attempted to find optimal conditons and solvent system was one of them</t>
+        </is>
+      </c>
     </row>
     <row r="185" ht="60" customHeight="1">
       <c r="A185" s="2" t="inlineStr">
@@ -10002,7 +10306,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J185" s="2" t="n"/>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>listed many screening conditions attempted to find optimal conditons and solvent system was one of them</t>
+        </is>
+      </c>
     </row>
     <row r="186" ht="60" customHeight="1">
       <c r="A186" s="2" t="inlineStr">
@@ -10052,7 +10360,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J186" s="2" t="n"/>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>listed many screening conditions attempted to find optimal conditons and solvent system was one of them</t>
+        </is>
+      </c>
     </row>
     <row r="187" ht="75" customHeight="1">
       <c r="A187" s="2" t="inlineStr">
@@ -10099,7 +10411,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J187" s="2" t="n"/>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="188" ht="60" customHeight="1">
       <c r="A188" s="2" t="inlineStr">
@@ -10145,7 +10461,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J188" s="2" t="n"/>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>says crystals of product could not be obtained for pH higher than 7 or lower than 6</t>
+        </is>
+      </c>
     </row>
     <row r="189" ht="60" customHeight="1">
       <c r="A189" s="2" t="inlineStr">
@@ -10191,7 +10511,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J189" s="2" t="n"/>
+      <c r="J189" s="2" t="inlineStr">
+        <is>
+          <t>says crystals of product could not be obtained for pH higher than 7 or lower than 6</t>
+        </is>
+      </c>
     </row>
     <row r="190" ht="75" customHeight="1">
       <c r="A190" s="2" t="inlineStr">
@@ -10238,7 +10562,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J190" s="2" t="n"/>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="191" ht="75" customHeight="1">
       <c r="A191" s="2" t="inlineStr">
@@ -10285,7 +10613,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J191" s="2" t="n"/>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="192" ht="75" customHeight="1">
       <c r="A192" s="2" t="inlineStr">
@@ -10332,7 +10664,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J192" s="2" t="n"/>
+      <c r="J192" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="193" ht="45" customHeight="1">
       <c r="A193" s="2" t="inlineStr">
@@ -10377,7 +10713,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J193" s="2" t="n"/>
+      <c r="J193" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="194" ht="45" customHeight="1">
       <c r="A194" s="2" t="inlineStr">
@@ -10422,7 +10762,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J194" s="2" t="n"/>
+      <c r="J194" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="195" ht="45" customHeight="1">
       <c r="A195" s="2" t="inlineStr">
@@ -10467,7 +10811,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J195" s="2" t="n"/>
+      <c r="J195" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="196" ht="45" customHeight="1">
       <c r="A196" s="2" t="inlineStr">
@@ -10512,7 +10860,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J196" s="2" t="n"/>
+      <c r="J196" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="197" ht="45" customHeight="1">
       <c r="A197" s="2" t="inlineStr">
@@ -10557,7 +10909,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J197" s="2" t="n"/>
+      <c r="J197" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="198" ht="45" customHeight="1">
       <c r="A198" s="2" t="inlineStr">
@@ -10602,7 +10958,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J198" s="2" t="n"/>
+      <c r="J198" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="199" ht="60" customHeight="1">
       <c r="A199" s="2" t="inlineStr">
@@ -10648,7 +11008,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J199" s="2" t="n"/>
+      <c r="J199" s="2" t="inlineStr">
+        <is>
+          <t>says crystals of product could not be obtained for pH higher than 7 or lower than 6</t>
+        </is>
+      </c>
     </row>
     <row r="200" ht="60" customHeight="1">
       <c r="A200" s="2" t="inlineStr">
@@ -10694,7 +11058,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J200" s="2" t="n"/>
+      <c r="J200" s="2" t="inlineStr">
+        <is>
+          <t>says crystals of product could not be obtained for pH higher than 7 or lower than 6</t>
+        </is>
+      </c>
     </row>
     <row r="201" ht="45" customHeight="1">
       <c r="A201" s="2" t="inlineStr">
@@ -10739,7 +11107,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J201" s="2" t="n"/>
+      <c r="J201" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="202" ht="60" customHeight="1">
       <c r="A202" s="2" t="inlineStr">
@@ -10785,7 +11157,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J202" s="2" t="n"/>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t>says crystals of product could not be obtained for pH higher than 7 or lower than 6</t>
+        </is>
+      </c>
     </row>
     <row r="203" ht="60" customHeight="1">
       <c r="A203" s="2" t="inlineStr">
@@ -10831,7 +11207,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J203" s="2" t="n"/>
+      <c r="J203" s="2" t="inlineStr">
+        <is>
+          <t>says crystals of product could not be obtained for pH higher than 7 or lower than 6</t>
+        </is>
+      </c>
     </row>
     <row r="204" ht="75" customHeight="1">
       <c r="A204" s="2" t="inlineStr">
@@ -10878,7 +11258,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J204" s="2" t="n"/>
+      <c r="J204" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="205" ht="75" customHeight="1">
       <c r="A205" s="2" t="inlineStr">
@@ -10925,7 +11309,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J205" s="2" t="n"/>
+      <c r="J205" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="206" ht="75" customHeight="1">
       <c r="A206" s="2" t="inlineStr">
@@ -10972,7 +11360,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J206" s="2" t="n"/>
+      <c r="J206" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="207" ht="75" customHeight="1">
       <c r="A207" s="2" t="inlineStr">
@@ -11019,7 +11411,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J207" s="2" t="n"/>
+      <c r="J207" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="208" ht="75" customHeight="1">
       <c r="A208" s="2" t="inlineStr">
@@ -11066,7 +11462,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J208" s="2" t="n"/>
+      <c r="J208" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="209" ht="60" customHeight="1">
       <c r="A209" s="2" t="inlineStr">
@@ -11112,7 +11512,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J209" s="2" t="n"/>
+      <c r="J209" s="2" t="inlineStr">
+        <is>
+          <t>says crystals of product could not be obtained for pH higher than 7 or lower than 6</t>
+        </is>
+      </c>
     </row>
     <row r="210" ht="60" customHeight="1">
       <c r="A210" s="2" t="inlineStr">
@@ -11158,7 +11562,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J210" s="2" t="n"/>
+      <c r="J210" s="2" t="inlineStr">
+        <is>
+          <t>says crystals of product could not be obtained for pH higher than 7 or lower than 6</t>
+        </is>
+      </c>
     </row>
     <row r="211" ht="75" customHeight="1">
       <c r="A211" s="2" t="inlineStr">
@@ -11205,7 +11613,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J211" s="2" t="n"/>
+      <c r="J211" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="212" ht="75" customHeight="1">
       <c r="A212" s="2" t="inlineStr">
@@ -11252,7 +11664,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J212" s="2" t="n"/>
+      <c r="J212" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="213" ht="75" customHeight="1">
       <c r="A213" s="2" t="inlineStr">
@@ -11299,7 +11715,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J213" s="2" t="n"/>
+      <c r="J213" s="2" t="inlineStr">
+        <is>
+          <t>lists a lot of M:L ratios as giving a few specific products and says all other ratios failed to produce products</t>
+        </is>
+      </c>
     </row>
     <row r="214" ht="45" customHeight="1">
       <c r="A214" s="2" t="inlineStr">
@@ -11348,7 +11768,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J214" s="2" t="n"/>
+      <c r="J214" s="2" t="inlineStr">
+        <is>
+          <t>lists other ligands and says that cannot recreate this crystal structue</t>
+        </is>
+      </c>
     </row>
     <row r="215" ht="45" customHeight="1">
       <c r="A215" s="2" t="inlineStr">
@@ -11397,7 +11821,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J215" s="2" t="n"/>
+      <c r="J215" s="2" t="inlineStr">
+        <is>
+          <t>lists other ligands and says that cannot recreate this crystal structue</t>
+        </is>
+      </c>
     </row>
     <row r="216" ht="45" customHeight="1">
       <c r="A216" s="2" t="inlineStr">
@@ -11446,7 +11874,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J216" s="2" t="n"/>
+      <c r="J216" s="2" t="inlineStr">
+        <is>
+          <t>lists other ligands and says that cannot recreate this crystal structue</t>
+        </is>
+      </c>
     </row>
     <row r="217" ht="45" customHeight="1">
       <c r="A217" s="2" t="inlineStr">
@@ -11495,7 +11927,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J217" s="2" t="n"/>
+      <c r="J217" s="2" t="inlineStr">
+        <is>
+          <t>lists other ligands and says that cannot recreate this crystal structue</t>
+        </is>
+      </c>
     </row>
     <row r="218" ht="45" customHeight="1">
       <c r="A218" s="2" t="inlineStr">
@@ -11544,7 +11980,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J218" s="2" t="n"/>
+      <c r="J218" s="2" t="inlineStr">
+        <is>
+          <t>says any attempts to recreate synthesis with a cadmium atom have not yet succeeded</t>
+        </is>
+      </c>
     </row>
     <row r="219" ht="38" customHeight="1">
       <c r="A219" s="3" t="inlineStr">
@@ -11631,7 +12071,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J220" s="2" t="n"/>
+      <c r="J220" s="2" t="inlineStr">
+        <is>
+          <t>addition of DMF shows remarkable loss o crystalinity</t>
+        </is>
+      </c>
     </row>
     <row r="221" ht="45" customHeight="1">
       <c r="A221" s="2" t="inlineStr">
@@ -11676,7 +12120,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J221" s="2" t="n"/>
+      <c r="J221" s="2" t="inlineStr">
+        <is>
+          <t>says solvothermal reactions of less than 24 H have minimal product</t>
+        </is>
+      </c>
     </row>
     <row r="222" ht="45" customHeight="1">
       <c r="A222" s="2" t="inlineStr">
@@ -11721,7 +12169,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J222" s="2" t="n"/>
+      <c r="J222" s="2" t="inlineStr">
+        <is>
+          <t>says solvothermal reactions of less than 24 H have minimal product</t>
+        </is>
+      </c>
     </row>
     <row r="223" ht="45" customHeight="1">
       <c r="A223" s="2" t="inlineStr">
@@ -11766,7 +12218,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J223" s="2" t="n"/>
+      <c r="J223" s="2" t="inlineStr">
+        <is>
+          <t>says solvothermal reactions of less than 24 H have minimal product</t>
+        </is>
+      </c>
     </row>
     <row r="224" ht="45" customHeight="1">
       <c r="A224" s="2" t="inlineStr">
@@ -11811,7 +12267,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J224" s="2" t="n"/>
+      <c r="J224" s="2" t="inlineStr">
+        <is>
+          <t>says solvothermal reactions of less than 24 H have minimal product</t>
+        </is>
+      </c>
     </row>
     <row r="225" ht="105" customHeight="1">
       <c r="A225" s="2" t="inlineStr">
@@ -11864,7 +12324,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J225" s="2" t="n"/>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t>says that at low overall concentations amorphous products were obtained, independatn of the amount of naoh added</t>
+        </is>
+      </c>
     </row>
     <row r="226" ht="105" customHeight="1">
       <c r="A226" s="2" t="inlineStr">
@@ -11917,7 +12381,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J226" s="2" t="n"/>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>says that at low overall concentations amorphous products were obtained, independatn of the amount of naoh added</t>
+        </is>
+      </c>
     </row>
     <row r="227" ht="105" customHeight="1">
       <c r="A227" s="2" t="inlineStr">
@@ -11970,7 +12438,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J227" s="2" t="n"/>
+      <c r="J227" s="2" t="inlineStr">
+        <is>
+          <t>says that at low overall concentations amorphous products were obtained, independatn of the amount of naoh added</t>
+        </is>
+      </c>
     </row>
     <row r="228" ht="120" customHeight="1">
       <c r="A228" s="2" t="inlineStr">
@@ -12024,7 +12496,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J228" s="2" t="n"/>
+      <c r="J228" s="2" t="inlineStr">
+        <is>
+          <t>said product was obtained at all moalr ratio without any noah, with naoh mix different products was found</t>
+        </is>
+      </c>
     </row>
     <row r="229" ht="120" customHeight="1">
       <c r="A229" s="2" t="inlineStr">
@@ -12078,7 +12554,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J229" s="2" t="n"/>
+      <c r="J229" s="2" t="inlineStr">
+        <is>
+          <t>said product was obtained at all moalr ratio without any noah, with naoh mix different products was found</t>
+        </is>
+      </c>
     </row>
     <row r="230" ht="120" customHeight="1">
       <c r="A230" s="2" t="inlineStr">
@@ -12132,7 +12612,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J230" s="2" t="n"/>
+      <c r="J230" s="2" t="inlineStr">
+        <is>
+          <t>said product was obtained at all moalr ratio without any noah, with naoh mix different products was found</t>
+        </is>
+      </c>
     </row>
     <row r="231" ht="135" customHeight="1">
       <c r="A231" s="2" t="inlineStr">
@@ -12187,7 +12671,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J231" s="2" t="n"/>
+      <c r="J231" s="2" t="inlineStr">
+        <is>
+          <t>said product was obtained at all moalr ratio without any noah, with naoh mix different products was found</t>
+        </is>
+      </c>
     </row>
     <row r="232" ht="135" customHeight="1">
       <c r="A232" s="2" t="inlineStr">
@@ -12242,7 +12730,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J232" s="2" t="n"/>
+      <c r="J232" s="2" t="inlineStr">
+        <is>
+          <t>said product was obtained at all moalr ratio without any noah, with naoh mix different products was found</t>
+        </is>
+      </c>
     </row>
     <row r="233" ht="135" customHeight="1">
       <c r="A233" s="2" t="inlineStr">
@@ -12297,7 +12789,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J233" s="2" t="n"/>
+      <c r="J233" s="2" t="inlineStr">
+        <is>
+          <t>said product was obtained at all moalr ratio without any noah, with naoh mix different products was found</t>
+        </is>
+      </c>
     </row>
     <row r="234" ht="45" customHeight="1">
       <c r="A234" s="2" t="inlineStr">
@@ -12346,7 +12842,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J234" s="2" t="n"/>
+      <c r="J234" s="2" t="inlineStr">
+        <is>
+          <t>says direct synthesis without a protecting group was not successful</t>
+        </is>
+      </c>
     </row>
     <row r="235" ht="60" customHeight="1">
       <c r="A235" s="2" t="inlineStr">
@@ -12392,7 +12892,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J235" s="2" t="n"/>
+      <c r="J235" s="2" t="inlineStr">
+        <is>
+          <t>says reaction in DMF or DEA without tea gives a 2d grid not MOF-5</t>
+        </is>
+      </c>
     </row>
     <row r="236" ht="60" customHeight="1">
       <c r="A236" s="2" t="inlineStr">
@@ -12438,7 +12942,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J236" s="2" t="n"/>
+      <c r="J236" s="2" t="inlineStr">
+        <is>
+          <t>says reaction in DMF or DEA without tea gives a 2d grid not MOF-5</t>
+        </is>
+      </c>
     </row>
     <row r="237" ht="45" customHeight="1">
       <c r="A237" s="2" t="inlineStr">
@@ -12487,7 +12995,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J237" s="2" t="n"/>
+      <c r="J237" s="2" t="inlineStr">
+        <is>
+          <t>says higher tesmos lead to decomposition and lower temps lead to less cryatline product</t>
+        </is>
+      </c>
     </row>
     <row r="238" ht="45" customHeight="1">
       <c r="A238" s="2" t="inlineStr">
@@ -12536,7 +13048,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J238" s="2" t="n"/>
+      <c r="J238" s="2" t="inlineStr">
+        <is>
+          <t>says higher tesmos lead to decomposition and lower temps lead to less cryatline product</t>
+        </is>
+      </c>
     </row>
     <row r="239" ht="45" customHeight="1">
       <c r="A239" s="2" t="inlineStr">
@@ -12581,7 +13097,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J239" s="2" t="n"/>
+      <c r="J239" s="2" t="inlineStr">
+        <is>
+          <t>says reactions at low temp gave amorphours material at low yield</t>
+        </is>
+      </c>
     </row>
     <row r="240" ht="60" customHeight="1">
       <c r="A240" s="2" t="inlineStr">
@@ -12627,7 +13147,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J240" s="2" t="n"/>
+      <c r="J240" s="2" t="inlineStr">
+        <is>
+          <t>says at high temps and with high zic rations prodcut contaiedn very little of comoound 7</t>
+        </is>
+      </c>
     </row>
     <row r="241" ht="45" customHeight="1">
       <c r="A241" s="2" t="inlineStr">
@@ -12672,7 +13196,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J241" s="2" t="n"/>
+      <c r="J241" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="242" ht="45" customHeight="1">
       <c r="A242" s="2" t="inlineStr">
@@ -12717,7 +13245,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J242" s="2" t="n"/>
+      <c r="J242" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="243" ht="45" customHeight="1">
       <c r="A243" s="2" t="inlineStr">
@@ -12762,7 +13294,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J243" s="2" t="n"/>
+      <c r="J243" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="244" ht="45" customHeight="1">
       <c r="A244" s="2" t="inlineStr">
@@ -12807,7 +13343,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J244" s="2" t="n"/>
+      <c r="J244" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="245" ht="45" customHeight="1">
       <c r="A245" s="2" t="inlineStr">
@@ -12852,7 +13392,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J245" s="2" t="n"/>
+      <c r="J245" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="246" ht="45" customHeight="1">
       <c r="A246" s="2" t="inlineStr">
@@ -12897,7 +13441,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J246" s="2" t="n"/>
+      <c r="J246" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="247" ht="45" customHeight="1">
       <c r="A247" s="2" t="inlineStr">
@@ -12942,7 +13490,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J247" s="2" t="n"/>
+      <c r="J247" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="248" ht="45" customHeight="1">
       <c r="A248" s="2" t="inlineStr">
@@ -12987,7 +13539,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J248" s="2" t="n"/>
+      <c r="J248" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="249" ht="45" customHeight="1">
       <c r="A249" s="2" t="inlineStr">
@@ -13032,7 +13588,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J249" s="2" t="n"/>
+      <c r="J249" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="250" ht="45" customHeight="1">
       <c r="A250" s="2" t="inlineStr">
@@ -13077,7 +13637,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J250" s="2" t="n"/>
+      <c r="J250" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="251" ht="45" customHeight="1">
       <c r="A251" s="2" t="inlineStr">
@@ -13122,7 +13686,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J251" s="2" t="n"/>
+      <c r="J251" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="252" ht="45" customHeight="1">
       <c r="A252" s="2" t="inlineStr">
@@ -13167,7 +13735,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J252" s="2" t="n"/>
+      <c r="J252" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="253" ht="60" customHeight="1">
       <c r="A253" s="2" t="inlineStr">
@@ -13217,7 +13789,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J253" s="2" t="n"/>
+      <c r="J253" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="254" ht="60" customHeight="1">
       <c r="A254" s="2" t="inlineStr">
@@ -13267,7 +13843,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J254" s="2" t="n"/>
+      <c r="J254" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="255" ht="60" customHeight="1">
       <c r="A255" s="2" t="inlineStr">
@@ -13317,7 +13897,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J255" s="2" t="n"/>
+      <c r="J255" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="256" ht="60" customHeight="1">
       <c r="A256" s="2" t="inlineStr">
@@ -13367,7 +13951,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J256" s="2" t="n"/>
+      <c r="J256" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="257" ht="60" customHeight="1">
       <c r="A257" s="2" t="inlineStr">
@@ -13417,7 +14005,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J257" s="2" t="n"/>
+      <c r="J257" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="258" ht="60" customHeight="1">
       <c r="A258" s="2" t="inlineStr">
@@ -13467,7 +14059,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J258" s="2" t="n"/>
+      <c r="J258" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="259" ht="60" customHeight="1">
       <c r="A259" s="2" t="inlineStr">
@@ -13517,7 +14113,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J259" s="2" t="n"/>
+      <c r="J259" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="260" ht="60" customHeight="1">
       <c r="A260" s="2" t="inlineStr">
@@ -13567,7 +14167,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J260" s="2" t="n"/>
+      <c r="J260" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="261" ht="60" customHeight="1">
       <c r="A261" s="2" t="inlineStr">
@@ -13617,7 +14221,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J261" s="2" t="n"/>
+      <c r="J261" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="262" ht="60" customHeight="1">
       <c r="A262" s="2" t="inlineStr">
@@ -13667,7 +14275,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J262" s="2" t="n"/>
+      <c r="J262" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="263" ht="75" customHeight="1">
       <c r="A263" s="2" t="inlineStr">
@@ -13718,7 +14330,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J263" s="2" t="n"/>
+      <c r="J263" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="264" ht="75" customHeight="1">
       <c r="A264" s="2" t="inlineStr">
@@ -13769,7 +14385,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J264" s="2" t="n"/>
+      <c r="J264" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="265" ht="75" customHeight="1">
       <c r="A265" s="2" t="inlineStr">
@@ -13820,7 +14440,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J265" s="2" t="n"/>
+      <c r="J265" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="266" ht="75" customHeight="1">
       <c r="A266" s="2" t="inlineStr">
@@ -13871,7 +14495,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J266" s="2" t="n"/>
+      <c r="J266" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="267" ht="75" customHeight="1">
       <c r="A267" s="2" t="inlineStr">
@@ -13922,7 +14550,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J267" s="2" t="n"/>
+      <c r="J267" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="268" ht="75" customHeight="1">
       <c r="A268" s="2" t="inlineStr">
@@ -13973,7 +14605,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J268" s="2" t="n"/>
+      <c r="J268" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="269" ht="75" customHeight="1">
       <c r="A269" s="2" t="inlineStr">
@@ -14024,7 +14660,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J269" s="2" t="n"/>
+      <c r="J269" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="270" ht="75" customHeight="1">
       <c r="A270" s="2" t="inlineStr">
@@ -14075,7 +14715,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J270" s="2" t="n"/>
+      <c r="J270" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="271" ht="75" customHeight="1">
       <c r="A271" s="2" t="inlineStr">
@@ -14126,7 +14770,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J271" s="2" t="n"/>
+      <c r="J271" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="272" ht="75" customHeight="1">
       <c r="A272" s="2" t="inlineStr">
@@ -14177,7 +14825,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J272" s="2" t="n"/>
+      <c r="J272" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="273" ht="90" customHeight="1">
       <c r="A273" s="2" t="inlineStr">
@@ -14229,7 +14881,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J273" s="2" t="n"/>
+      <c r="J273" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="274" ht="90" customHeight="1">
       <c r="A274" s="2" t="inlineStr">
@@ -14281,7 +14937,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J274" s="2" t="n"/>
+      <c r="J274" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="275" ht="90" customHeight="1">
       <c r="A275" s="2" t="inlineStr">
@@ -14333,7 +14993,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J275" s="2" t="n"/>
+      <c r="J275" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="276" ht="90" customHeight="1">
       <c r="A276" s="2" t="inlineStr">
@@ -14385,7 +15049,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J276" s="2" t="n"/>
+      <c r="J276" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="277" ht="90" customHeight="1">
       <c r="A277" s="2" t="inlineStr">
@@ -14437,7 +15105,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J277" s="2" t="n"/>
+      <c r="J277" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="278" ht="105" customHeight="1">
       <c r="A278" s="2" t="inlineStr">
@@ -14490,7 +15162,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J278" s="2" t="n"/>
+      <c r="J278" s="2" t="inlineStr">
+        <is>
+          <t>says compounds 5 and 6(precursors) were reacted with a few zinc salts and a few different solvents at various stoichiometries, mainly leading to amorphous or microcrysaltine powders</t>
+        </is>
+      </c>
     </row>
     <row r="279" ht="45" customHeight="1">
       <c r="A279" s="2" t="inlineStr">
@@ -14539,7 +15215,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J279" s="2" t="n"/>
+      <c r="J279" s="2" t="inlineStr">
+        <is>
+          <t>says using naoh instead of dbu lead to the formation of a low crystaline phase</t>
+        </is>
+      </c>
     </row>
     <row r="280" ht="150" customHeight="1">
       <c r="A280" s="2" t="inlineStr">
@@ -14595,7 +15275,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J280" s="2" t="n"/>
+      <c r="J280" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13</t>
+        </is>
+      </c>
     </row>
     <row r="281" ht="135" customHeight="1">
       <c r="A281" s="2" t="inlineStr">
@@ -14650,7 +15334,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J281" s="2" t="n"/>
+      <c r="J281" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13</t>
+        </is>
+      </c>
     </row>
     <row r="282" ht="135" customHeight="1">
       <c r="A282" s="2" t="inlineStr">
@@ -14705,7 +15393,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J282" s="2" t="n"/>
+      <c r="J282" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13</t>
+        </is>
+      </c>
     </row>
     <row r="283" ht="135" customHeight="1">
       <c r="A283" s="2" t="inlineStr">
@@ -14760,7 +15452,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J283" s="2" t="n"/>
+      <c r="J283" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13</t>
+        </is>
+      </c>
     </row>
     <row r="284" ht="150" customHeight="1">
       <c r="A284" s="2" t="inlineStr">
@@ -14816,7 +15512,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J284" s="2" t="n"/>
+      <c r="J284" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13</t>
+        </is>
+      </c>
     </row>
     <row r="285" ht="150" customHeight="1">
       <c r="A285" s="2" t="inlineStr">
@@ -14872,7 +15572,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J285" s="2" t="n"/>
+      <c r="J285" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13</t>
+        </is>
+      </c>
     </row>
     <row r="286" ht="150" customHeight="1">
       <c r="A286" s="2" t="inlineStr">
@@ -14928,7 +15632,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J286" s="2" t="n"/>
+      <c r="J286" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13</t>
+        </is>
+      </c>
     </row>
     <row r="287" ht="150" customHeight="1">
       <c r="A287" s="2" t="inlineStr">
@@ -14984,7 +15692,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J287" s="2" t="n"/>
+      <c r="J287" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13</t>
+        </is>
+      </c>
     </row>
     <row r="288" ht="120" customHeight="1">
       <c r="A288" s="2" t="inlineStr">
@@ -15038,7 +15750,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J288" s="2" t="n"/>
+      <c r="J288" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13</t>
+        </is>
+      </c>
     </row>
     <row r="289" ht="120" customHeight="1">
       <c r="A289" s="2" t="inlineStr">
@@ -15092,7 +15808,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J289" s="2" t="n"/>
+      <c r="J289" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13</t>
+        </is>
+      </c>
     </row>
     <row r="290" ht="120" customHeight="1">
       <c r="A290" s="2" t="inlineStr">
@@ -15146,7 +15866,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J290" s="2" t="n"/>
+      <c r="J290" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13 and s14</t>
+        </is>
+      </c>
     </row>
     <row r="291" ht="120" customHeight="1">
       <c r="A291" s="2" t="inlineStr">
@@ -15200,7 +15924,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J291" s="2" t="n"/>
+      <c r="J291" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13 and s14</t>
+        </is>
+      </c>
     </row>
     <row r="292" ht="120" customHeight="1">
       <c r="A292" s="2" t="inlineStr">
@@ -15254,7 +15982,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J292" s="2" t="n"/>
+      <c r="J292" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13 and s14</t>
+        </is>
+      </c>
     </row>
     <row r="293" ht="150" customHeight="1">
       <c r="A293" s="2" t="inlineStr">
@@ -15310,7 +16042,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J293" s="2" t="n"/>
+      <c r="J293" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13 and s14</t>
+        </is>
+      </c>
     </row>
     <row r="294" ht="135" customHeight="1">
       <c r="A294" s="2" t="inlineStr">
@@ -15365,7 +16101,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J294" s="2" t="n"/>
+      <c r="J294" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13 and s14</t>
+        </is>
+      </c>
     </row>
     <row r="295" ht="135" customHeight="1">
       <c r="A295" s="2" t="inlineStr">
@@ -15420,7 +16160,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J295" s="2" t="n"/>
+      <c r="J295" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13 and s14</t>
+        </is>
+      </c>
     </row>
     <row r="296" ht="135" customHeight="1">
       <c r="A296" s="2" t="inlineStr">
@@ -15475,7 +16219,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J296" s="2" t="n"/>
+      <c r="J296" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13 and s14</t>
+        </is>
+      </c>
     </row>
     <row r="297" ht="150" customHeight="1">
       <c r="A297" s="2" t="inlineStr">
@@ -15531,7 +16279,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J297" s="2" t="n"/>
+      <c r="J297" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13 and s14</t>
+        </is>
+      </c>
     </row>
     <row r="298" ht="150" customHeight="1">
       <c r="A298" s="2" t="inlineStr">
@@ -15587,7 +16339,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J298" s="2" t="n"/>
+      <c r="J298" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13 and s14</t>
+        </is>
+      </c>
     </row>
     <row r="299" ht="150" customHeight="1">
       <c r="A299" s="2" t="inlineStr">
@@ -15643,7 +16399,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J299" s="2" t="n"/>
+      <c r="J299" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13 and s14</t>
+        </is>
+      </c>
     </row>
     <row r="300" ht="135" customHeight="1">
       <c r="A300" s="2" t="inlineStr">
@@ -15698,7 +16458,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J300" s="2" t="n"/>
+      <c r="J300" s="2" t="inlineStr">
+        <is>
+          <t>Screening reactions shown with results in table S12 and S13 and s14</t>
+        </is>
+      </c>
     </row>
     <row r="301" ht="75" customHeight="1">
       <c r="A301" s="2" t="inlineStr">
@@ -15749,7 +16513,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J301" s="2" t="n"/>
+      <c r="J301" s="2" t="inlineStr">
+        <is>
+          <t>says reaction without hcl did not work</t>
+        </is>
+      </c>
     </row>
     <row r="302" ht="75" customHeight="1">
       <c r="A302" s="2" t="inlineStr">
@@ -15800,7 +16568,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J302" s="2" t="n"/>
+      <c r="J302" s="2" t="inlineStr">
+        <is>
+          <t>says using zr oac as a precusor under high concentrations gave poorly crystaline material</t>
+        </is>
+      </c>
     </row>
     <row r="303" ht="45" customHeight="1">
       <c r="A303" s="2" t="inlineStr">
@@ -15849,7 +16621,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J303" s="2" t="n"/>
+      <c r="J303" s="2" t="inlineStr">
+        <is>
+          <t>mof formation using zrpiv requried 72 hours</t>
+        </is>
+      </c>
     </row>
     <row r="304" ht="45" customHeight="1">
       <c r="A304" s="2" t="inlineStr">
@@ -15898,7 +16674,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J304" s="2" t="n"/>
+      <c r="J304" s="2" t="inlineStr">
+        <is>
+          <t>mof formation using zrpiv requried 72 hours</t>
+        </is>
+      </c>
     </row>
     <row r="305" ht="45" customHeight="1">
       <c r="A305" s="2" t="inlineStr">
@@ -15947,7 +16727,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J305" s="2" t="n"/>
+      <c r="J305" s="2" t="inlineStr">
+        <is>
+          <t>high concentrations of linker lead to poorly crystaline mateiral</t>
+        </is>
+      </c>
     </row>
     <row r="306" ht="45" customHeight="1">
       <c r="A306" s="2" t="inlineStr">
@@ -15996,7 +16780,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J306" s="2" t="n"/>
+      <c r="J306" s="2" t="inlineStr">
+        <is>
+          <t>high concentrations of linker lead to poorly crystaline mateiral</t>
+        </is>
+      </c>
     </row>
     <row r="307" ht="45" customHeight="1">
       <c r="A307" s="2" t="inlineStr">
@@ -16045,7 +16833,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J307" s="2" t="n"/>
+      <c r="J307" s="2" t="inlineStr">
+        <is>
+          <t>says the use of carboxilic acid to replace hcl to form MOF product was essential, in either case no modulator leads to fail</t>
+        </is>
+      </c>
     </row>
     <row r="308" ht="135" customHeight="1">
       <c r="A308" s="2" t="inlineStr">
@@ -16100,7 +16892,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J308" s="2" t="n"/>
+      <c r="J308" s="2" t="inlineStr">
+        <is>
+          <t>unsuccessful ball milling synth</t>
+        </is>
+      </c>
     </row>
     <row r="309" ht="135" customHeight="1">
       <c r="A309" s="2" t="inlineStr">
@@ -16155,7 +16951,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J309" s="2" t="n"/>
+      <c r="J309" s="2" t="inlineStr">
+        <is>
+          <t>unsuccessful ball milling synth</t>
+        </is>
+      </c>
     </row>
     <row r="310" ht="45" customHeight="1">
       <c r="A310" s="2" t="inlineStr">
@@ -16204,7 +17004,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J310" s="2" t="n"/>
+      <c r="J310" s="2" t="inlineStr">
+        <is>
+          <t>says the use of carboxilic acid to replace hcl to form MOF product was essential, in either case no modulator leads to fail</t>
+        </is>
+      </c>
     </row>
     <row r="311" ht="45" customHeight="1">
       <c r="A311" s="2" t="inlineStr">
@@ -16253,7 +17057,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J311" s="2" t="n"/>
+      <c r="J311" s="2" t="inlineStr">
+        <is>
+          <t>says the use of carboxilic acid to replace hcl to form MOF product was essential, in either case no modulator leads to fail</t>
+        </is>
+      </c>
     </row>
     <row r="312" ht="135" customHeight="1">
       <c r="A312" s="2" t="inlineStr">
@@ -16308,7 +17116,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J312" s="2" t="n"/>
+      <c r="J312" s="2" t="inlineStr">
+        <is>
+          <t>unsuccessful ball milling synth</t>
+        </is>
+      </c>
     </row>
     <row r="313" ht="135" customHeight="1">
       <c r="A313" s="2" t="inlineStr">
@@ -16363,7 +17175,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J313" s="2" t="n"/>
+      <c r="J313" s="2" t="inlineStr">
+        <is>
+          <t>unsuccessful ball milling synth</t>
+        </is>
+      </c>
     </row>
     <row r="314" ht="45" customHeight="1">
       <c r="A314" s="2" t="inlineStr">
@@ -16412,7 +17228,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J314" s="2" t="n"/>
+      <c r="J314" s="2" t="inlineStr">
+        <is>
+          <t>says the use of carboxilic acid to replace hcl to form MOF product was essential, in either case no modulator leads to fail</t>
+        </is>
+      </c>
     </row>
     <row r="315" ht="38" customHeight="1">
       <c r="A315" s="3" t="inlineStr">
@@ -16542,7 +17362,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J317" s="2" t="n"/>
+      <c r="J317" s="2" t="inlineStr">
+        <is>
+          <t>screening tables list condtions with no mof formed</t>
+        </is>
+      </c>
     </row>
     <row r="318" ht="45" customHeight="1">
       <c r="A318" s="2" t="inlineStr">
@@ -16591,7 +17415,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J318" s="2" t="n"/>
+      <c r="J318" s="2" t="inlineStr">
+        <is>
+          <t>screening tables list condtions with no mof formed</t>
+        </is>
+      </c>
     </row>
     <row r="319" ht="45" customHeight="1">
       <c r="A319" s="2" t="inlineStr">
@@ -16640,7 +17468,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J319" s="2" t="n"/>
+      <c r="J319" s="2" t="inlineStr">
+        <is>
+          <t>SI table SI shows with no naOH there is no signifigant percipitation</t>
+        </is>
+      </c>
     </row>
     <row r="320" ht="60" customHeight="1">
       <c r="A320" s="2" t="inlineStr">
@@ -16690,7 +17522,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J320" s="2" t="n"/>
+      <c r="J320" s="2" t="inlineStr">
+        <is>
+          <t>Si table S1 shows results with failed perciptates</t>
+        </is>
+      </c>
     </row>
     <row r="321" ht="45" customHeight="1">
       <c r="A321" s="2" t="inlineStr">
@@ -16739,7 +17575,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J321" s="2" t="n"/>
+      <c r="J321" s="2" t="inlineStr">
+        <is>
+          <t>table  S1 shown no tea yields failed reactions</t>
+        </is>
+      </c>
     </row>
     <row r="322" ht="60" customHeight="1">
       <c r="A322" s="2" t="inlineStr">
@@ -16789,7 +17629,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J322" s="2" t="n"/>
+      <c r="J322" s="2" t="inlineStr">
+        <is>
+          <t>mof cannot be made in pure alccohols</t>
+        </is>
+      </c>
     </row>
     <row r="323" ht="60" customHeight="1">
       <c r="A323" s="2" t="inlineStr">
@@ -16839,7 +17683,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J323" s="2" t="n"/>
+      <c r="J323" s="2" t="inlineStr">
+        <is>
+          <t>mof cannot be made in pure alccohols</t>
+        </is>
+      </c>
     </row>
     <row r="324" ht="60" customHeight="1">
       <c r="A324" s="2" t="inlineStr">
@@ -16889,7 +17737,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J324" s="2" t="n"/>
+      <c r="J324" s="2" t="inlineStr">
+        <is>
+          <t>mof cannot be made in pure alccohols</t>
+        </is>
+      </c>
     </row>
     <row r="325" ht="60" customHeight="1">
       <c r="A325" s="2" t="inlineStr">
@@ -16939,7 +17791,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J325" s="2" t="n"/>
+      <c r="J325" s="2" t="inlineStr">
+        <is>
+          <t>mof cannot be made in pure alccohols</t>
+        </is>
+      </c>
     </row>
     <row r="326" ht="60" customHeight="1">
       <c r="A326" s="2" t="inlineStr">
@@ -16989,7 +17845,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J326" s="2" t="n"/>
+      <c r="J326" s="2" t="inlineStr">
+        <is>
+          <t>mof cannot be made in pure alccohols</t>
+        </is>
+      </c>
     </row>
     <row r="327" ht="60" customHeight="1">
       <c r="A327" s="2" t="inlineStr">
@@ -17039,7 +17899,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J327" s="2" t="n"/>
+      <c r="J327" s="2" t="inlineStr">
+        <is>
+          <t>mof cannot be made in pure alccohols</t>
+        </is>
+      </c>
     </row>
     <row r="328" ht="75" customHeight="1">
       <c r="A328" s="2" t="inlineStr">
@@ -17090,7 +17954,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J328" s="2" t="n"/>
+      <c r="J328" s="2" t="inlineStr">
+        <is>
+          <t>table s2 shows screening reactions with modulator</t>
+        </is>
+      </c>
     </row>
     <row r="329" ht="75" customHeight="1">
       <c r="A329" s="2" t="inlineStr">
@@ -17141,7 +18009,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J329" s="2" t="n"/>
+      <c r="J329" s="2" t="inlineStr">
+        <is>
+          <t>table s2 shows screening reactions with modulator</t>
+        </is>
+      </c>
     </row>
     <row r="330" ht="75" customHeight="1">
       <c r="A330" s="2" t="inlineStr">
@@ -17192,7 +18064,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J330" s="2" t="n"/>
+      <c r="J330" s="2" t="inlineStr">
+        <is>
+          <t>table s2 shows screening reactions with modulator</t>
+        </is>
+      </c>
     </row>
     <row r="331" ht="75" customHeight="1">
       <c r="A331" s="2" t="inlineStr">
@@ -17243,7 +18119,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J331" s="2" t="n"/>
+      <c r="J331" s="2" t="inlineStr">
+        <is>
+          <t>table s2 shows screening reactions with modulator</t>
+        </is>
+      </c>
     </row>
     <row r="332" ht="105" customHeight="1">
       <c r="A332" s="2" t="inlineStr">
@@ -17296,7 +18176,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J332" s="2" t="n"/>
+      <c r="J332" s="2" t="inlineStr">
+        <is>
+          <t>table s3 shows screening reactions with temp, time</t>
+        </is>
+      </c>
     </row>
     <row r="333" ht="120" customHeight="1">
       <c r="A333" s="2" t="inlineStr">
@@ -17350,7 +18234,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J333" s="2" t="n"/>
+      <c r="J333" s="2" t="inlineStr">
+        <is>
+          <t>table s3 shows screening reactions with temp, time</t>
+        </is>
+      </c>
     </row>
     <row r="334" ht="120" customHeight="1">
       <c r="A334" s="2" t="inlineStr">
@@ -17404,7 +18292,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J334" s="2" t="n"/>
+      <c r="J334" s="2" t="inlineStr">
+        <is>
+          <t>table s3 shows screening reactions with temp, time</t>
+        </is>
+      </c>
     </row>
     <row r="335" ht="120" customHeight="1">
       <c r="A335" s="2" t="inlineStr">
@@ -17458,7 +18350,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J335" s="2" t="n"/>
+      <c r="J335" s="2" t="inlineStr">
+        <is>
+          <t>table s3 shows screening reactions with temp, time</t>
+        </is>
+      </c>
     </row>
     <row r="336" ht="120" customHeight="1">
       <c r="A336" s="2" t="inlineStr">
@@ -17512,7 +18408,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J336" s="2" t="n"/>
+      <c r="J336" s="2" t="inlineStr">
+        <is>
+          <t>table s3 shows screening reactions with temp, time</t>
+        </is>
+      </c>
     </row>
     <row r="337" ht="75" customHeight="1">
       <c r="A337" s="2" t="inlineStr">
@@ -17563,7 +18463,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J337" s="2" t="n"/>
+      <c r="J337" s="2" t="inlineStr">
+        <is>
+          <t>table s2 shows screening reactions with temp, time</t>
+        </is>
+      </c>
     </row>
     <row r="338" ht="75" customHeight="1">
       <c r="A338" s="2" t="inlineStr">
@@ -17614,7 +18518,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J338" s="2" t="n"/>
+      <c r="J338" s="2" t="inlineStr">
+        <is>
+          <t>table s2 shows screening reactions with temp, time</t>
+        </is>
+      </c>
     </row>
     <row r="339" ht="60" customHeight="1">
       <c r="A339" s="2" t="inlineStr">
@@ -17664,7 +18572,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J339" s="2" t="n"/>
+      <c r="J339" s="2" t="inlineStr">
+        <is>
+          <t>table s2 shows screening reactions with temp, time</t>
+        </is>
+      </c>
     </row>
     <row r="340" ht="60" customHeight="1">
       <c r="A340" s="2" t="inlineStr">
@@ -17714,7 +18626,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J340" s="2" t="n"/>
+      <c r="J340" s="2" t="inlineStr">
+        <is>
+          <t>table s2 shows screening reactions with temp, time</t>
+        </is>
+      </c>
     </row>
     <row r="341" ht="60" customHeight="1">
       <c r="A341" s="2" t="inlineStr">
@@ -17764,7 +18680,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J341" s="2" t="n"/>
+      <c r="J341" s="2" t="inlineStr">
+        <is>
+          <t>table s2 shows screening reactions with temp, time</t>
+        </is>
+      </c>
     </row>
     <row r="342" ht="60" customHeight="1">
       <c r="A342" s="2" t="inlineStr">
@@ -17814,7 +18734,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J342" s="2" t="n"/>
+      <c r="J342" s="2" t="inlineStr">
+        <is>
+          <t>table s2 shows screening reactions with temp, time</t>
+        </is>
+      </c>
     </row>
     <row r="343" ht="45" customHeight="1">
       <c r="A343" s="2" t="inlineStr">
@@ -17859,7 +18783,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J343" s="2" t="n"/>
+      <c r="J343" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="344" ht="45" customHeight="1">
       <c r="A344" s="2" t="inlineStr">
@@ -17904,7 +18832,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J344" s="2" t="n"/>
+      <c r="J344" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="345" ht="45" customHeight="1">
       <c r="A345" s="2" t="inlineStr">
@@ -17949,7 +18881,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J345" s="2" t="n"/>
+      <c r="J345" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="346" ht="45" customHeight="1">
       <c r="A346" s="2" t="inlineStr">
@@ -17994,7 +18930,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J346" s="2" t="n"/>
+      <c r="J346" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="347" ht="45" customHeight="1">
       <c r="A347" s="2" t="inlineStr">
@@ -18039,7 +18979,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J347" s="2" t="n"/>
+      <c r="J347" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="348" ht="45" customHeight="1">
       <c r="A348" s="2" t="inlineStr">
@@ -18084,7 +19028,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J348" s="2" t="n"/>
+      <c r="J348" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="349" ht="45" customHeight="1">
       <c r="A349" s="2" t="inlineStr">
@@ -18129,7 +19077,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J349" s="2" t="n"/>
+      <c r="J349" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="350" ht="45" customHeight="1">
       <c r="A350" s="2" t="inlineStr">
@@ -18174,7 +19126,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J350" s="2" t="n"/>
+      <c r="J350" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="351" ht="45" customHeight="1">
       <c r="A351" s="2" t="inlineStr">
@@ -18219,7 +19175,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J351" s="2" t="n"/>
+      <c r="J351" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="352" ht="45" customHeight="1">
       <c r="A352" s="2" t="inlineStr">
@@ -18264,7 +19224,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J352" s="2" t="n"/>
+      <c r="J352" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="353" ht="45" customHeight="1">
       <c r="A353" s="2" t="inlineStr">
@@ -18309,7 +19273,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J353" s="2" t="n"/>
+      <c r="J353" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="354" ht="45" customHeight="1">
       <c r="A354" s="2" t="inlineStr">
@@ -18354,7 +19322,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J354" s="2" t="n"/>
+      <c r="J354" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="355" ht="45" customHeight="1">
       <c r="A355" s="2" t="inlineStr">
@@ -18399,7 +19371,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J355" s="2" t="n"/>
+      <c r="J355" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="356" ht="45" customHeight="1">
       <c r="A356" s="2" t="inlineStr">
@@ -18444,7 +19420,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J356" s="2" t="n"/>
+      <c r="J356" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="357" ht="45" customHeight="1">
       <c r="A357" s="2" t="inlineStr">
@@ -18489,7 +19469,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J357" s="2" t="n"/>
+      <c r="J357" s="2" t="inlineStr">
+        <is>
+          <t>shows that other acids fail to yield a product</t>
+        </is>
+      </c>
     </row>
     <row r="358" ht="45" customHeight="1">
       <c r="A358" s="2" t="inlineStr">
@@ -18538,7 +19522,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J358" s="2" t="n"/>
+      <c r="J358" s="2" t="inlineStr">
+        <is>
+          <t>was difficult to obtain solid product without bpe</t>
+        </is>
+      </c>
     </row>
     <row r="359" ht="45" customHeight="1">
       <c r="A359" s="2" t="inlineStr">
@@ -18587,7 +19575,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J359" s="2" t="n"/>
+      <c r="J359" s="2" t="inlineStr">
+        <is>
+          <t>h2o said to be umportant to high quality crystal, amorphous without it</t>
+        </is>
+      </c>
     </row>
     <row r="360" ht="45" customHeight="1">
       <c r="A360" s="2" t="inlineStr">
@@ -18636,7 +19628,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J360" s="2" t="n"/>
+      <c r="J360" s="2" t="inlineStr">
+        <is>
+          <t>h2o said to be umportant to high quality crystal, amorphous without it</t>
+        </is>
+      </c>
     </row>
     <row r="361" ht="45" customHeight="1">
       <c r="A361" s="2" t="inlineStr">
@@ -18685,7 +19681,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J361" s="2" t="n"/>
+      <c r="J361" s="2" t="inlineStr">
+        <is>
+          <t>h2o said to be umportant to high quality crystal, amorphous without it</t>
+        </is>
+      </c>
     </row>
     <row r="362" ht="60" customHeight="1">
       <c r="A362" s="2" t="inlineStr">
@@ -18735,7 +19735,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J362" s="2" t="n"/>
+      <c r="J362" s="2" t="inlineStr">
+        <is>
+          <t>above .5 mmol naoac charactizlation lines of pxrd vanihs, mof desotryed</t>
+        </is>
+      </c>
     </row>
     <row r="363" ht="60" customHeight="1">
       <c r="A363" s="2" t="inlineStr">
@@ -18785,7 +19789,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J363" s="2" t="n"/>
+      <c r="J363" s="2" t="inlineStr">
+        <is>
+          <t>above .5 mmol naoac charactizlation lines of pxrd vanihs, mof desotryed</t>
+        </is>
+      </c>
     </row>
     <row r="364" ht="60" customHeight="1">
       <c r="A364" s="2" t="inlineStr">
@@ -18835,7 +19843,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J364" s="2" t="n"/>
+      <c r="J364" s="2" t="inlineStr">
+        <is>
+          <t>above .5 mmol naoac charactizlation lines of pxrd vanihs, mof desotryed</t>
+        </is>
+      </c>
     </row>
     <row r="365" ht="38" customHeight="1">
       <c r="A365" s="3" t="inlineStr">
@@ -18925,7 +19937,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J366" s="2" t="n"/>
+      <c r="J366" s="2" t="inlineStr">
+        <is>
+          <t>co-im system made inorganic side products not normal mof</t>
+        </is>
+      </c>
     </row>
     <row r="367" ht="60" customHeight="1">
       <c r="A367" s="2" t="inlineStr">
@@ -18975,7 +19991,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J367" s="2" t="n"/>
+      <c r="J367" s="2" t="inlineStr">
+        <is>
+          <t>co-im system made inorganic side products not normal mof</t>
+        </is>
+      </c>
     </row>
     <row r="368" ht="60" customHeight="1">
       <c r="A368" s="2" t="inlineStr">
@@ -19025,7 +20045,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J368" s="2" t="n"/>
+      <c r="J368" s="2" t="inlineStr">
+        <is>
+          <t>co-im system made inorganic side products not normal mof</t>
+        </is>
+      </c>
     </row>
     <row r="369" ht="60" customHeight="1">
       <c r="A369" s="2" t="inlineStr">
@@ -19075,7 +20099,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J369" s="2" t="n"/>
+      <c r="J369" s="2" t="inlineStr">
+        <is>
+          <t>co-im system made inorganic side products not normal mof</t>
+        </is>
+      </c>
     </row>
     <row r="370" ht="60" customHeight="1">
       <c r="A370" s="2" t="inlineStr">
@@ -19125,7 +20153,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J370" s="2" t="n"/>
+      <c r="J370" s="2" t="inlineStr">
+        <is>
+          <t>co-im system made inorganic side products not normal mof</t>
+        </is>
+      </c>
     </row>
     <row r="371" ht="60" customHeight="1">
       <c r="A371" s="2" t="inlineStr">
@@ -19175,7 +20207,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J371" s="2" t="n"/>
+      <c r="J371" s="2" t="inlineStr">
+        <is>
+          <t>co-im system made inorganic side products not normal mof</t>
+        </is>
+      </c>
     </row>
     <row r="372" ht="38" customHeight="1">
       <c r="A372" s="3" t="inlineStr">
@@ -19309,7 +20345,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J374" s="2" t="n"/>
+      <c r="J374" s="2" t="inlineStr">
+        <is>
+          <t>paragraph of screening conditions to make new products yielded failed conditons until ionic liquid precusor was used</t>
+        </is>
+      </c>
     </row>
     <row r="375" ht="120" customHeight="1">
       <c r="A375" s="2" t="inlineStr">
@@ -19363,7 +20403,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J375" s="2" t="n"/>
+      <c r="J375" s="2" t="inlineStr">
+        <is>
+          <t>paragraph of screening conditions to make new products yielded failed conditons until ionic liquid precusor was used</t>
+        </is>
+      </c>
     </row>
     <row r="376" ht="120" customHeight="1">
       <c r="A376" s="2" t="inlineStr">
@@ -19417,7 +20461,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J376" s="2" t="n"/>
+      <c r="J376" s="2" t="inlineStr">
+        <is>
+          <t>paragraph of screening conditions to make new products yielded failed conditons until ionic liquid precusor was used</t>
+        </is>
+      </c>
     </row>
     <row r="377" ht="45" customHeight="1">
       <c r="A377" s="2" t="inlineStr">
@@ -19462,7 +20510,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J377" s="2" t="n"/>
+      <c r="J377" s="2" t="inlineStr">
+        <is>
+          <t>lists solvents as attempted but failed</t>
+        </is>
+      </c>
     </row>
     <row r="378" ht="45" customHeight="1">
       <c r="A378" s="2" t="inlineStr">
@@ -19507,7 +20559,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J378" s="2" t="n"/>
+      <c r="J378" s="2" t="inlineStr">
+        <is>
+          <t>lists solvents as attempted but failed</t>
+        </is>
+      </c>
     </row>
     <row r="379" ht="45" customHeight="1">
       <c r="A379" s="2" t="inlineStr">
@@ -19552,7 +20608,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J379" s="2" t="n"/>
+      <c r="J379" s="2" t="inlineStr">
+        <is>
+          <t>lists solvents as attempted but failed</t>
+        </is>
+      </c>
     </row>
     <row r="380" ht="45" customHeight="1">
       <c r="A380" s="2" t="inlineStr">
@@ -19597,7 +20657,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J380" s="2" t="n"/>
+      <c r="J380" s="2" t="inlineStr">
+        <is>
+          <t>lists solvents as attempted but failed</t>
+        </is>
+      </c>
     </row>
     <row r="381" ht="45" customHeight="1">
       <c r="A381" s="2" t="inlineStr">
@@ -19642,7 +20706,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J381" s="2" t="n"/>
+      <c r="J381" s="2" t="inlineStr">
+        <is>
+          <t>lists solvents as attempted but failed</t>
+        </is>
+      </c>
     </row>
     <row r="382" ht="45" customHeight="1">
       <c r="A382" s="2" t="inlineStr">
@@ -19687,7 +20755,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J382" s="2" t="n"/>
+      <c r="J382" s="2" t="inlineStr">
+        <is>
+          <t>lists solvents as attempted but failed</t>
+        </is>
+      </c>
     </row>
     <row r="383" ht="45" customHeight="1">
       <c r="A383" s="2" t="inlineStr">
@@ -19732,7 +20804,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J383" s="2" t="n"/>
+      <c r="J383" s="2" t="inlineStr">
+        <is>
+          <t>direct synthesis of copper analog was not successful</t>
+        </is>
+      </c>
     </row>
     <row r="384" ht="45" customHeight="1">
       <c r="A384" s="2" t="inlineStr">
@@ -19781,7 +20857,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J384" s="2" t="n"/>
+      <c r="J384" s="2" t="inlineStr">
+        <is>
+          <t>introducing the L proline results in a sharp decrease of crystalinity</t>
+        </is>
+      </c>
     </row>
     <row r="385" ht="45" customHeight="1">
       <c r="A385" s="2" t="inlineStr">
@@ -19830,7 +20910,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J385" s="2" t="n"/>
+      <c r="J385" s="2" t="inlineStr">
+        <is>
+          <t>found that heating at 100 C yieldied amorphous substances</t>
+        </is>
+      </c>
     </row>
     <row r="386" ht="38" customHeight="1">
       <c r="A386" s="3" t="inlineStr">
@@ -19920,7 +21004,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J387" s="2" t="n"/>
+      <c r="J387" s="2" t="inlineStr">
+        <is>
+          <t>paper says crystals cannot be obtained when more than 3 eq HF added</t>
+        </is>
+      </c>
     </row>
     <row r="388" ht="60" customHeight="1">
       <c r="A388" s="2" t="inlineStr">
@@ -19966,7 +21054,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J388" s="2" t="n"/>
+      <c r="J388" s="2" t="inlineStr">
+        <is>
+          <t>says many metal salts formed h3lno3 instead of coordination networks</t>
+        </is>
+      </c>
     </row>
     <row r="389" ht="45" customHeight="1">
       <c r="A389" s="2" t="inlineStr">
@@ -20011,7 +21103,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J389" s="2" t="n"/>
+      <c r="J389" s="2" t="inlineStr">
+        <is>
+          <t>says many metal salts formed h3lno3 instead of coordination networks</t>
+        </is>
+      </c>
     </row>
     <row r="390" ht="45" customHeight="1">
       <c r="A390" s="2" t="inlineStr">
@@ -20056,7 +21152,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J390" s="2" t="n"/>
+      <c r="J390" s="2" t="inlineStr">
+        <is>
+          <t>says when amount of base was increased only unknown deposits were obtained</t>
+        </is>
+      </c>
     </row>
     <row r="391" ht="45" customHeight="1">
       <c r="A391" s="2" t="inlineStr">
@@ -20101,7 +21201,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J391" s="2" t="n"/>
+      <c r="J391" s="2" t="inlineStr">
+        <is>
+          <t>says when amount of base was increased only unknown deposits were obtained</t>
+        </is>
+      </c>
     </row>
     <row r="392" ht="45" customHeight="1">
       <c r="A392" s="2" t="inlineStr">
@@ -20146,7 +21250,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J392" s="2" t="n"/>
+      <c r="J392" s="2" t="inlineStr">
+        <is>
+          <t>says when amount of base was increased only unknown deposits were obtained</t>
+        </is>
+      </c>
     </row>
     <row r="393" ht="45" customHeight="1">
       <c r="A393" s="2" t="inlineStr">
@@ -20191,7 +21299,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J393" s="2" t="n"/>
+      <c r="J393" s="2" t="inlineStr">
+        <is>
+          <t>says when amount of base was increased only unknown deposits were obtained</t>
+        </is>
+      </c>
     </row>
     <row r="394" ht="45" customHeight="1">
       <c r="A394" s="2" t="inlineStr">
@@ -20240,7 +21352,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J394" s="2" t="n"/>
+      <c r="J394" s="2" t="inlineStr">
+        <is>
+          <t>when no hcl was used products with irregular shapes and weak diffractions peaks were obtained</t>
+        </is>
+      </c>
     </row>
     <row r="395" ht="75" customHeight="1">
       <c r="A395" s="2" t="inlineStr">
@@ -20291,7 +21407,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J395" s="2" t="n"/>
+      <c r="J395" s="2" t="inlineStr">
+        <is>
+          <t>with no hcl a concentration screening was permfored and under a cetain ratios no products were made</t>
+        </is>
+      </c>
     </row>
     <row r="396" ht="75" customHeight="1">
       <c r="A396" s="2" t="inlineStr">
@@ -20342,7 +21462,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J396" s="2" t="n"/>
+      <c r="J396" s="2" t="inlineStr">
+        <is>
+          <t>with no hcl a concentration screening was permfored and under a cetain ratios no products were made</t>
+        </is>
+      </c>
     </row>
     <row r="397" ht="75" customHeight="1">
       <c r="A397" s="2" t="inlineStr">
@@ -20393,7 +21517,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J397" s="2" t="n"/>
+      <c r="J397" s="2" t="inlineStr">
+        <is>
+          <t>at certain ratios a blue precipitate</t>
+        </is>
+      </c>
     </row>
     <row r="398" ht="60" customHeight="1">
       <c r="A398" s="2" t="inlineStr">
@@ -20443,7 +21571,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J398" s="2" t="n"/>
+      <c r="J398" s="2" t="inlineStr">
+        <is>
+          <t>tea played a vital role in regularing the uniformity of building units, other sdas were attempted but did not work</t>
+        </is>
+      </c>
     </row>
     <row r="399" ht="60" customHeight="1">
       <c r="A399" s="2" t="inlineStr">
@@ -20493,7 +21625,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J399" s="2" t="n"/>
+      <c r="J399" s="2" t="inlineStr">
+        <is>
+          <t>tea played a vital role in regularing the uniformity of building units, other sdas were attempted but did not work</t>
+        </is>
+      </c>
     </row>
     <row r="400" ht="60" customHeight="1">
       <c r="A400" s="2" t="inlineStr">
@@ -20543,7 +21679,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J400" s="2" t="n"/>
+      <c r="J400" s="2" t="inlineStr">
+        <is>
+          <t>tea played a vital role in regularing the uniformity of building units, other sdas were attempted but did not work</t>
+        </is>
+      </c>
     </row>
     <row r="401" ht="60" customHeight="1">
       <c r="A401" s="2" t="inlineStr">
@@ -20593,7 +21733,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J401" s="2" t="n"/>
+      <c r="J401" s="2" t="inlineStr">
+        <is>
+          <t>use of modulator said to be critical for formation of polymof</t>
+        </is>
+      </c>
     </row>
     <row r="402" ht="45" customHeight="1">
       <c r="A402" s="2" t="inlineStr">
@@ -20642,7 +21786,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J402" s="2" t="n"/>
+      <c r="J402" s="2" t="inlineStr">
+        <is>
+          <t>said pbdc-10a-u folred amorpjhous mateirals in filmss</t>
+        </is>
+      </c>
     </row>
     <row r="403" ht="60" customHeight="1">
       <c r="A403" s="2" t="inlineStr">
@@ -20692,7 +21840,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J403" s="2" t="n"/>
+      <c r="J403" s="2" t="inlineStr">
+        <is>
+          <t>use of modulator said to be critical for formation of polymof</t>
+        </is>
+      </c>
     </row>
     <row r="404" ht="60" customHeight="1">
       <c r="A404" s="2" t="inlineStr">
@@ -20742,7 +21894,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J404" s="2" t="n"/>
+      <c r="J404" s="2" t="inlineStr">
+        <is>
+          <t>use of modulator said to be critical for formation of polymof</t>
+        </is>
+      </c>
     </row>
     <row r="405" ht="45" customHeight="1">
       <c r="A405" s="2" t="inlineStr">
@@ -20791,7 +21947,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J405" s="2" t="n"/>
+      <c r="J405" s="2" t="inlineStr">
+        <is>
+          <t>only pbdc-xa only works with x=3-8+</t>
+        </is>
+      </c>
     </row>
     <row r="406" ht="45" customHeight="1">
       <c r="A406" s="2" t="inlineStr">
@@ -20840,7 +22000,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J406" s="2" t="n"/>
+      <c r="J406" s="2" t="inlineStr">
+        <is>
+          <t>only pbdc-xa only works with x=3-8+</t>
+        </is>
+      </c>
     </row>
     <row r="407" ht="60" customHeight="1">
       <c r="A407" s="2" t="inlineStr">
@@ -20890,7 +22054,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J407" s="2" t="n"/>
+      <c r="J407" s="2" t="inlineStr">
+        <is>
+          <t>use of modulator said to be critical for formation of polymof</t>
+        </is>
+      </c>
     </row>
     <row r="408" ht="45" customHeight="1">
       <c r="A408" s="2" t="inlineStr">
@@ -20935,7 +22103,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J408" s="2" t="n"/>
+      <c r="J408" s="2" t="inlineStr">
+        <is>
+          <t>no sucessful case for NaI and LiI ions</t>
+        </is>
+      </c>
     </row>
     <row r="409" ht="45" customHeight="1">
       <c r="A409" s="2" t="inlineStr">
@@ -20980,7 +22152,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J409" s="2" t="n"/>
+      <c r="J409" s="2" t="inlineStr">
+        <is>
+          <t>no sucessful case for NaI and LiI ions</t>
+        </is>
+      </c>
     </row>
     <row r="410" ht="45" customHeight="1">
       <c r="A410" s="2" t="inlineStr">
@@ -21025,7 +22201,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J410" s="2" t="n"/>
+      <c r="J410" s="2" t="inlineStr">
+        <is>
+          <t>no sucessful case for NaI and LiI ions</t>
+        </is>
+      </c>
     </row>
     <row r="411" ht="45" customHeight="1">
       <c r="A411" s="2" t="inlineStr">
@@ -21070,7 +22250,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J411" s="2" t="n"/>
+      <c r="J411" s="2" t="inlineStr">
+        <is>
+          <t>no sucessful case for NaI and LiI ions</t>
+        </is>
+      </c>
     </row>
     <row r="412" ht="45" customHeight="1">
       <c r="A412" s="2" t="inlineStr">
@@ -21115,7 +22299,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J412" s="2" t="n"/>
+      <c r="J412" s="2" t="inlineStr">
+        <is>
+          <t>no sucessful case for NaI and LiI ions</t>
+        </is>
+      </c>
     </row>
     <row r="413" ht="45" customHeight="1">
       <c r="A413" s="2" t="inlineStr">
@@ -21160,7 +22348,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J413" s="2" t="n"/>
+      <c r="J413" s="2" t="inlineStr">
+        <is>
+          <t>no sucessful case for NaI and LiI ions</t>
+        </is>
+      </c>
     </row>
     <row r="414" ht="45" customHeight="1">
       <c r="A414" s="2" t="inlineStr">
@@ -21205,7 +22397,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J414" s="2" t="n"/>
+      <c r="J414" s="2" t="inlineStr">
+        <is>
+          <t>no sucessful case for NaI and LiI ions</t>
+        </is>
+      </c>
     </row>
     <row r="415" ht="45" customHeight="1">
       <c r="A415" s="2" t="inlineStr">
@@ -21250,7 +22446,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J415" s="2" t="n"/>
+      <c r="J415" s="2" t="inlineStr">
+        <is>
+          <t>no sucessful case for NaI and LiI ions</t>
+        </is>
+      </c>
     </row>
     <row r="416" ht="75" customHeight="1">
       <c r="A416" s="2" t="inlineStr">
@@ -21301,7 +22501,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J416" s="2" t="n"/>
+      <c r="J416" s="2" t="inlineStr">
+        <is>
+          <t>created nonprous coordination polymer not MOF</t>
+        </is>
+      </c>
     </row>
     <row r="417" ht="45" customHeight="1">
       <c r="A417" s="2" t="inlineStr">
@@ -21350,7 +22554,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J417" s="2" t="n"/>
+      <c r="J417" s="2" t="inlineStr">
+        <is>
+          <t>with no hac xrd peaks were greatly diminished</t>
+        </is>
+      </c>
     </row>
     <row r="418" ht="60" customHeight="1">
       <c r="A418" s="2" t="inlineStr">
@@ -21400,7 +22608,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J418" s="2" t="n"/>
+      <c r="J418" s="2" t="inlineStr">
+        <is>
+          <t>products decrease In crystalinity and temp is lowered</t>
+        </is>
+      </c>
     </row>
     <row r="419" ht="45" customHeight="1">
       <c r="A419" s="2" t="inlineStr">
@@ -21449,7 +22661,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J419" s="2" t="n"/>
+      <c r="J419" s="2" t="inlineStr">
+        <is>
+          <t>reagents were insoluble in THF at low temperatures</t>
+        </is>
+      </c>
     </row>
     <row r="420" ht="45" customHeight="1">
       <c r="A420" s="2" t="inlineStr">
@@ -21498,7 +22714,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J420" s="2" t="n"/>
+      <c r="J420" s="2" t="inlineStr">
+        <is>
+          <t>if the free thiol pf htt is directly mixed with metal, amorphous percipiate is formed</t>
+        </is>
+      </c>
     </row>
     <row r="421" ht="60" customHeight="1">
       <c r="A421" s="2" t="inlineStr">
@@ -21548,7 +22768,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J421" s="2" t="n"/>
+      <c r="J421" s="2" t="inlineStr">
+        <is>
+          <t>if the free thiol pf htt is directly mixed with metal, amorphous percipiate is formed even at longer reaction times</t>
+        </is>
+      </c>
     </row>
     <row r="422" ht="45" customHeight="1">
       <c r="A422" s="2" t="inlineStr">
@@ -21593,7 +22817,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J422" s="2" t="n"/>
+      <c r="J422" s="2" t="inlineStr">
+        <is>
+          <t>showed a large collection of linkers and said all except 1 but nothing could be formed except percipitate</t>
+        </is>
+      </c>
     </row>
     <row r="423" ht="60" customHeight="1">
       <c r="A423" s="2" t="inlineStr">
@@ -21639,7 +22867,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J423" s="2" t="n"/>
+      <c r="J423" s="2" t="inlineStr">
+        <is>
+          <t>showed a large collection of linkers and said all except 1 but nothing could be formed except percipitate</t>
+        </is>
+      </c>
     </row>
     <row r="424" ht="45" customHeight="1">
       <c r="A424" s="2" t="inlineStr">
@@ -21684,7 +22916,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J424" s="2" t="n"/>
+      <c r="J424" s="2" t="inlineStr">
+        <is>
+          <t>showed a large collection of linkers and said all except 1 but nothing could be formed except percipitate</t>
+        </is>
+      </c>
     </row>
     <row r="425" ht="45" customHeight="1">
       <c r="A425" s="2" t="inlineStr">
@@ -21733,7 +22969,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J425" s="2" t="n"/>
+      <c r="J425" s="2" t="inlineStr">
+        <is>
+          <t>the use of alcohols, dmf or thf leads to only very low yields of the MOF</t>
+        </is>
+      </c>
     </row>
     <row r="426" ht="45" customHeight="1">
       <c r="A426" s="2" t="inlineStr">
@@ -21782,7 +23022,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J426" s="2" t="n"/>
+      <c r="J426" s="2" t="inlineStr">
+        <is>
+          <t>the use of alcohols, dmf or thf leads to only very low yields of the MOF</t>
+        </is>
+      </c>
     </row>
     <row r="427" ht="45" customHeight="1">
       <c r="A427" s="2" t="inlineStr">
@@ -21831,7 +23075,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J427" s="2" t="n"/>
+      <c r="J427" s="2" t="inlineStr">
+        <is>
+          <t>the use of alcohols, dmf or thf leads to only very low yields of the MOF</t>
+        </is>
+      </c>
     </row>
     <row r="428" ht="90" customHeight="1">
       <c r="A428" s="2" t="inlineStr">
@@ -21883,7 +23131,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J428" s="2" t="n"/>
+      <c r="J428" s="2" t="inlineStr">
+        <is>
+          <t>at pH 14 the oxide is the major product according to PXRD</t>
+        </is>
+      </c>
     </row>
     <row r="429" ht="60" customHeight="1">
       <c r="A429" s="2" t="inlineStr">
@@ -21933,7 +23185,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J429" s="2" t="n"/>
+      <c r="J429" s="2" t="inlineStr">
+        <is>
+          <t>the use of 0 and 12 eq naoh resulted in xray amorphous products</t>
+        </is>
+      </c>
     </row>
     <row r="430" ht="45" customHeight="1">
       <c r="A430" s="2" t="inlineStr">
@@ -21982,7 +23238,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J430" s="2" t="n"/>
+      <c r="J430" s="2" t="inlineStr">
+        <is>
+          <t>a metal to linker ratio of 1:1 resulting in low crystalinity</t>
+        </is>
+      </c>
     </row>
     <row r="431" ht="60" customHeight="1">
       <c r="A431" s="2" t="inlineStr">
@@ -22032,7 +23292,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J431" s="2" t="n"/>
+      <c r="J431" s="2" t="inlineStr">
+        <is>
+          <t>says various addatives were tried buyt only NaF with NaOh resulted in the formation of product</t>
+        </is>
+      </c>
     </row>
     <row r="432" ht="60" customHeight="1">
       <c r="A432" s="2" t="inlineStr">
@@ -22082,7 +23346,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J432" s="2" t="n"/>
+      <c r="J432" s="2" t="inlineStr">
+        <is>
+          <t>says various addatives were tried buyt only NaF with NaOh resulted in the formation of product</t>
+        </is>
+      </c>
     </row>
     <row r="433" ht="60" customHeight="1">
       <c r="A433" s="2" t="inlineStr">
@@ -22132,7 +23400,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J433" s="2" t="n"/>
+      <c r="J433" s="2" t="inlineStr">
+        <is>
+          <t>says various addatives were tried buyt only NaF with NaOh resulted in the formation of product</t>
+        </is>
+      </c>
     </row>
     <row r="434" ht="60" customHeight="1">
       <c r="A434" s="2" t="inlineStr">
@@ -22182,7 +23454,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J434" s="2" t="n"/>
+      <c r="J434" s="2" t="inlineStr">
+        <is>
+          <t>says various addatives were tried buyt only NaF with NaOh resulted in the formation of product</t>
+        </is>
+      </c>
     </row>
     <row r="435" ht="60" customHeight="1">
       <c r="A435" s="2" t="inlineStr">
@@ -22232,7 +23508,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J435" s="2" t="n"/>
+      <c r="J435" s="2" t="inlineStr">
+        <is>
+          <t>the use of 0 and 12 eq naoh resulted in xray amorphous products</t>
+        </is>
+      </c>
     </row>
     <row r="436" ht="45" customHeight="1">
       <c r="A436" s="2" t="inlineStr">
@@ -22281,7 +23561,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J436" s="2" t="n"/>
+      <c r="J436" s="2" t="inlineStr">
+        <is>
+          <t>a metal to linker ratio of 1:1 resulting in low crystalinity</t>
+        </is>
+      </c>
     </row>
     <row r="437" ht="60" customHeight="1">
       <c r="A437" s="2" t="inlineStr">
@@ -22331,7 +23615,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J437" s="2" t="n"/>
+      <c r="J437" s="2" t="inlineStr">
+        <is>
+          <t>says various addatives were tried buyt only NaF with NaOh resulted in the formation of product</t>
+        </is>
+      </c>
     </row>
     <row r="438" ht="60" customHeight="1">
       <c r="A438" s="2" t="inlineStr">
@@ -22381,7 +23669,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J438" s="2" t="n"/>
+      <c r="J438" s="2" t="inlineStr">
+        <is>
+          <t>says various addatives were tried buyt only NaF with NaOh resulted in the formation of product</t>
+        </is>
+      </c>
     </row>
     <row r="439" ht="60" customHeight="1">
       <c r="A439" s="2" t="inlineStr">
@@ -22431,7 +23723,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J439" s="2" t="n"/>
+      <c r="J439" s="2" t="inlineStr">
+        <is>
+          <t>says various addatives were tried buyt only NaF with NaOh resulted in the formation of product</t>
+        </is>
+      </c>
     </row>
     <row r="440" ht="60" customHeight="1">
       <c r="A440" s="2" t="inlineStr">
@@ -22481,7 +23777,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J440" s="2" t="n"/>
+      <c r="J440" s="2" t="inlineStr">
+        <is>
+          <t>says various addatives were tried buyt only NaF with NaOh resulted in the formation of product</t>
+        </is>
+      </c>
     </row>
     <row r="441" ht="75" customHeight="1">
       <c r="A441" s="2" t="inlineStr">
@@ -22532,7 +23832,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J441" s="2" t="n"/>
+      <c r="J441" s="2" t="inlineStr">
+        <is>
+          <t>exact conditions were stated for the unopimtized reaction compared to optimzied</t>
+        </is>
+      </c>
     </row>
     <row r="442" ht="45" customHeight="1">
       <c r="A442" s="2" t="inlineStr">
@@ -22581,7 +23885,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J442" s="2" t="n"/>
+      <c r="J442" s="2" t="inlineStr">
+        <is>
+          <t>said that after longer reaction times the title compound could not be obtained as pure product</t>
+        </is>
+      </c>
     </row>
     <row r="443" ht="45" customHeight="1">
       <c r="A443" s="2" t="inlineStr">
@@ -22630,7 +23938,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J443" s="2" t="n"/>
+      <c r="J443" s="2" t="inlineStr">
+        <is>
+          <t>said that after longer reaction times the title compound could not be obtained as pure product</t>
+        </is>
+      </c>
     </row>
     <row r="444" ht="45" customHeight="1">
       <c r="A444" s="2" t="inlineStr">
@@ -22679,7 +23991,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J444" s="2" t="n"/>
+      <c r="J444" s="2" t="inlineStr">
+        <is>
+          <t>said that after longer reaction times the title compound could not be obtained as pure product</t>
+        </is>
+      </c>
     </row>
     <row r="445" ht="45" customHeight="1">
       <c r="A445" s="2" t="inlineStr">
@@ -22728,7 +24044,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J445" s="2" t="n"/>
+      <c r="J445" s="2" t="inlineStr">
+        <is>
+          <t>when zinc nitrate was introduced instead of zinc acetate zif-f could not be synthesized</t>
+        </is>
+      </c>
     </row>
     <row r="446" ht="60" customHeight="1">
       <c r="A446" s="2" t="inlineStr">
@@ -22778,7 +24098,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J446" s="2" t="n"/>
+      <c r="J446" s="2" t="inlineStr">
+        <is>
+          <t>said that atfer 1 H a specific crystal was formed, and 1H later it converted to zif-8</t>
+        </is>
+      </c>
     </row>
     <row r="447" ht="60" customHeight="1">
       <c r="A447" s="2" t="inlineStr">
@@ -22828,7 +24152,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J447" s="2" t="n"/>
+      <c r="J447" s="2" t="inlineStr">
+        <is>
+          <t>said that atfer 1 H a specific crystal was formed, and 1H later it converted to zif-8</t>
+        </is>
+      </c>
     </row>
     <row r="448" ht="60" customHeight="1">
       <c r="A448" s="2" t="inlineStr">
@@ -22878,7 +24206,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J448" s="2" t="n"/>
+      <c r="J448" s="2" t="inlineStr">
+        <is>
+          <t>said that atfer 1 H a specific crystal was formed, and 1H later it converted to zif-8</t>
+        </is>
+      </c>
     </row>
     <row r="449" ht="45" customHeight="1">
       <c r="A449" s="2" t="inlineStr">
@@ -22927,7 +24259,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J449" s="2" t="n"/>
+      <c r="J449" s="2" t="inlineStr">
+        <is>
+          <t>says 1 metal procudure works but does not allow incorperating any doping metal by simply adding a second salt along with fecl2</t>
+        </is>
+      </c>
     </row>
     <row r="450" ht="45" customHeight="1">
       <c r="A450" s="2" t="inlineStr">
@@ -22976,7 +24312,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J450" s="2" t="n"/>
+      <c r="J450" s="2" t="inlineStr">
+        <is>
+          <t>says 1 metal procudure works but does not allow incorperating any doping metal by simply adding a second salt along with fecl2</t>
+        </is>
+      </c>
     </row>
     <row r="451" ht="45" customHeight="1">
       <c r="A451" s="2" t="inlineStr">
@@ -23025,7 +24365,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J451" s="2" t="n"/>
+      <c r="J451" s="2" t="inlineStr">
+        <is>
+          <t>says 1 metal procudure works but does not allow incorperating any doping metal by simply adding a second salt along with fecl2</t>
+        </is>
+      </c>
     </row>
     <row r="452" ht="45" customHeight="1">
       <c r="A452" s="2" t="inlineStr">
@@ -23074,7 +24418,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J452" s="2" t="n"/>
+      <c r="J452" s="2" t="inlineStr">
+        <is>
+          <t>says that pb2+ and bi3+ are not suitable for incorporation into mil-100(fe)</t>
+        </is>
+      </c>
     </row>
     <row r="453" ht="45" customHeight="1">
       <c r="A453" s="2" t="inlineStr">
@@ -23123,7 +24471,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J453" s="2" t="n"/>
+      <c r="J453" s="2" t="inlineStr">
+        <is>
+          <t>says that pb2+ and bi3+ are not suitable for incorporation into mil-100(fe)</t>
+        </is>
+      </c>
     </row>
     <row r="454" ht="45" customHeight="1">
       <c r="A454" s="2" t="inlineStr">
@@ -23172,7 +24524,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J454" s="2" t="n"/>
+      <c r="J454" s="2" t="inlineStr">
+        <is>
+          <t>says that pb2+ and bi3+ are not suitable for incorporation into mil-100(fe)</t>
+        </is>
+      </c>
     </row>
     <row r="455" ht="45" customHeight="1">
       <c r="A455" s="2" t="inlineStr">
@@ -23221,7 +24577,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J455" s="2" t="n"/>
+      <c r="J455" s="2" t="inlineStr">
+        <is>
+          <t>says that pb2+ and bi3+ are not suitable for incorporation into mil-100(fe)</t>
+        </is>
+      </c>
     </row>
     <row r="456" ht="45" customHeight="1">
       <c r="A456" s="2" t="inlineStr">
@@ -23270,7 +24630,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J456" s="2" t="n"/>
+      <c r="J456" s="2" t="inlineStr">
+        <is>
+          <t>says that pb2+ and bi3+ are not suitable for incorporation into mil-100(fe)</t>
+        </is>
+      </c>
     </row>
     <row r="457" ht="45" customHeight="1">
       <c r="A457" s="2" t="inlineStr">
@@ -23319,7 +24683,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J457" s="2" t="n"/>
+      <c r="J457" s="2" t="inlineStr">
+        <is>
+          <t>says that pb2+ and bi3+ are not suitable for incorporation into mil-100(fe)</t>
+        </is>
+      </c>
     </row>
     <row r="458" ht="60" customHeight="1">
       <c r="A458" s="2" t="inlineStr">
@@ -23369,7 +24737,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J458" s="2" t="n"/>
+      <c r="J458" s="2" t="inlineStr">
+        <is>
+          <t>says that iron chloride cant work for making crystals</t>
+        </is>
+      </c>
     </row>
     <row r="459" ht="60" customHeight="1">
       <c r="A459" s="2" t="inlineStr">
@@ -23419,7 +24791,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J459" s="2" t="n"/>
+      <c r="J459" s="2" t="inlineStr">
+        <is>
+          <t>says that iron chloride cant work for making crystals</t>
+        </is>
+      </c>
     </row>
     <row r="460" ht="60" customHeight="1">
       <c r="A460" s="2" t="inlineStr">
@@ -23469,7 +24845,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J460" s="2" t="n"/>
+      <c r="J460" s="2" t="inlineStr">
+        <is>
+          <t>says that iron chloride cant work for making crystals</t>
+        </is>
+      </c>
     </row>
     <row r="461" ht="60" customHeight="1">
       <c r="A461" s="2" t="inlineStr">
@@ -23519,7 +24899,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J461" s="2" t="n"/>
+      <c r="J461" s="2" t="inlineStr">
+        <is>
+          <t>said single crystals couldn’t be obtained with single monocarboxylic acid</t>
+        </is>
+      </c>
     </row>
     <row r="462" ht="60" customHeight="1">
       <c r="A462" s="2" t="inlineStr">
@@ -23569,7 +24953,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J462" s="2" t="n"/>
+      <c r="J462" s="2" t="inlineStr">
+        <is>
+          <t>said single crystals couldn’t be obtained with single monocarboxylic acid</t>
+        </is>
+      </c>
     </row>
     <row r="463" ht="60" customHeight="1">
       <c r="A463" s="2" t="inlineStr">
@@ -23619,7 +25007,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J463" s="2" t="n"/>
+      <c r="J463" s="2" t="inlineStr">
+        <is>
+          <t>said single crystals couldn’t be obtained with single monocarboxylic acid</t>
+        </is>
+      </c>
     </row>
     <row r="464" ht="60" customHeight="1">
       <c r="A464" s="2" t="inlineStr">
@@ -23669,7 +25061,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J464" s="2" t="n"/>
+      <c r="J464" s="2" t="inlineStr">
+        <is>
+          <t>says that iron chloride cant work for making crystals</t>
+        </is>
+      </c>
     </row>
     <row r="465" ht="45" customHeight="1">
       <c r="A465" s="2" t="inlineStr">
@@ -23714,7 +25110,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J465" s="2" t="n"/>
+      <c r="J465" s="2" t="inlineStr">
+        <is>
+          <t>said that by increasing or decraing temp framework cant be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="466" ht="45" customHeight="1">
       <c r="A466" s="2" t="inlineStr">
@@ -23759,7 +25159,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J466" s="2" t="n"/>
+      <c r="J466" s="2" t="inlineStr">
+        <is>
+          <t>said that by increasing or decraing temp framework cant be obtained</t>
+        </is>
+      </c>
     </row>
     <row r="467" ht="45" customHeight="1">
       <c r="A467" s="2" t="inlineStr">
@@ -23804,7 +25208,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J467" s="2" t="n"/>
+      <c r="J467" s="2" t="inlineStr">
+        <is>
+          <t>said that replacing with ina ligand to replace ligand cannot make target materials</t>
+        </is>
+      </c>
     </row>
     <row r="468" ht="45" customHeight="1">
       <c r="A468" s="2" t="inlineStr">
@@ -23849,7 +25257,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J468" s="2" t="n"/>
+      <c r="J468" s="2" t="inlineStr">
+        <is>
+          <t>using other copper saltsaaffects the quality of the crystals</t>
+        </is>
+      </c>
     </row>
     <row r="469" ht="45" customHeight="1">
       <c r="A469" s="2" t="inlineStr">
@@ -23894,7 +25306,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J469" s="2" t="n"/>
+      <c r="J469" s="2" t="inlineStr">
+        <is>
+          <t>using other copper saltsaaffects the quality of the crystals</t>
+        </is>
+      </c>
     </row>
     <row r="470" ht="45" customHeight="1">
       <c r="A470" s="2" t="inlineStr">
@@ -23939,7 +25355,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J470" s="2" t="n"/>
+      <c r="J470" s="2" t="inlineStr">
+        <is>
+          <t>using other copper saltsaaffects the quality of the crystals</t>
+        </is>
+      </c>
     </row>
     <row r="471" ht="45" customHeight="1">
       <c r="A471" s="2" t="inlineStr">
@@ -23984,7 +25404,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J471" s="2" t="n"/>
+      <c r="J471" s="2" t="inlineStr">
+        <is>
+          <t>using naoh as modulator yielded only na3ptc crystals</t>
+        </is>
+      </c>
     </row>
     <row r="472" ht="45" customHeight="1">
       <c r="A472" s="2" t="inlineStr">
@@ -24033,7 +25457,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J472" s="2" t="n"/>
+      <c r="J472" s="2" t="inlineStr">
+        <is>
+          <t>gu-3 and gu-4 were much less crystaline than gu-2</t>
+        </is>
+      </c>
     </row>
     <row r="473" ht="45" customHeight="1">
       <c r="A473" s="2" t="inlineStr">
@@ -24082,7 +25510,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J473" s="2" t="n"/>
+      <c r="J473" s="2" t="inlineStr">
+        <is>
+          <t>gu-3 and gu-4 were much less crystaline than gu-2</t>
+        </is>
+      </c>
     </row>
     <row r="474" ht="60" customHeight="1">
       <c r="A474" s="2" t="inlineStr">
@@ -24132,7 +25564,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J474" s="2" t="n"/>
+      <c r="J474" s="2" t="inlineStr">
+        <is>
+          <t>said attempts using other modulators were unsuscessfull</t>
+        </is>
+      </c>
     </row>
     <row r="475" ht="60" customHeight="1">
       <c r="A475" s="2" t="inlineStr">
@@ -24182,7 +25618,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J475" s="2" t="n"/>
+      <c r="J475" s="2" t="inlineStr">
+        <is>
+          <t>said attempts using other modulators were unsuscessfull</t>
+        </is>
+      </c>
     </row>
     <row r="476" ht="60" customHeight="1">
       <c r="A476" s="2" t="inlineStr">
@@ -24232,7 +25672,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J476" s="2" t="n"/>
+      <c r="J476" s="2" t="inlineStr">
+        <is>
+          <t>said attempts using other modulators were unsuscessfull</t>
+        </is>
+      </c>
     </row>
     <row r="477" ht="60" customHeight="1">
       <c r="A477" s="2" t="inlineStr">
@@ -24282,7 +25726,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J477" s="2" t="n"/>
+      <c r="J477" s="2" t="inlineStr">
+        <is>
+          <t>said attempts using other modulators were unsuscessfull</t>
+        </is>
+      </c>
     </row>
     <row r="478" ht="45" customHeight="1">
       <c r="A478" s="2" t="inlineStr">
@@ -24331,7 +25779,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J478" s="2" t="n"/>
+      <c r="J478" s="2" t="inlineStr">
+        <is>
+          <t>says at 50 C the reaction was incomplete</t>
+        </is>
+      </c>
     </row>
     <row r="479" ht="45" customHeight="1">
       <c r="A479" s="2" t="inlineStr">
@@ -24380,7 +25832,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J479" s="2" t="n"/>
+      <c r="J479" s="2" t="inlineStr">
+        <is>
+          <t>says over 60 yields no solid products due to overreduction of maganese</t>
+        </is>
+      </c>
     </row>
     <row r="480" ht="60" customHeight="1">
       <c r="A480" s="2" t="inlineStr">
@@ -24430,7 +25886,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J480" s="2" t="n"/>
+      <c r="J480" s="2" t="inlineStr">
+        <is>
+          <t>reports trying other modulators but no product was obtained</t>
+        </is>
+      </c>
     </row>
     <row r="481" ht="45" customHeight="1">
       <c r="A481" s="2" t="inlineStr">
@@ -24479,7 +25939,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J481" s="2" t="n"/>
+      <c r="J481" s="2" t="inlineStr">
+        <is>
+          <t>says the l2 ligand and long bpdc crysatline was never isolated into product</t>
+        </is>
+      </c>
     </row>
     <row r="482" ht="45" customHeight="1">
       <c r="A482" s="2" t="inlineStr">
@@ -24528,7 +25992,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="J482" s="2" t="n"/>
+      <c r="J482" s="2" t="inlineStr">
+        <is>
+          <t>says the l2 ligand and long bpdc crysatline was never isolated into product</t>
+        </is>
+      </c>
     </row>
     <row r="483" ht="38" customHeight="1">
       <c r="A483" s="3" t="inlineStr">

</xml_diff>